<commit_message>
Regenerate master translations workbook (v2, 545 labels) + summary update
Re-extracted every label from the platform after the Heritage Studio
replacement: 215 I18N keys + 330 inline bilingual strings (14 dynamic).
Updated PROJECT_SUMMARY.md to reflect the implemented/rejected ideas
and the new studio architecture notes.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CLDXbGK8zj9ZJ8qdP9uGRX
</commit_message>
<xml_diff>
--- a/TRANSLATIONS_MASTER.xlsx
+++ b/TRANSLATIONS_MASTER.xlsx
@@ -406,7 +406,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>📖 دليل استخدام ملف المسميات الشامل</v>
+        <v>📖 دليل استخدام ملف المسميات الشامل — الإصدار 2 (بعد استوديو التراث)</v>
       </c>
     </row>
     <row r="2">
@@ -416,7 +416,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>هذا الملف يحتوي حرفياً على كل نص يظهر على المنصة (603 مسمى) موزعة على ورقتين:</v>
+        <v>هذا الملف يحتوي حرفياً على كل نص يظهر على المنصة (545 مسمى) موزعة على ورقتين:</v>
       </c>
     </row>
     <row r="4">
@@ -431,7 +431,7 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>🟨 ورقة "2- نصوص مضمنة": نصوص الميزات المتقدمة (388) — تُحدد بنصها الحالي نفسه.</v>
+        <v>🟨 ورقة "2- نصوص مضمنة": نصوص الميزات المتقدمة والاستوديو (330) — تُحدد بنصها الحالي نفسه.</v>
       </c>
     </row>
     <row r="7">
@@ -4183,7 +4183,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F389"/>
+  <dimension ref="A1:F331"/>
   <cols>
     <col min="1" max="1" width="7.83203125" customWidth="1"/>
     <col min="2" max="2" width="60.83203125" customWidth="1"/>
@@ -6538,10 +6538,10 @@
         <v>T117</v>
       </c>
       <c r="B118" t="str">
-        <v>مركز البيانات المتقدم</v>
+        <v>استوديو التراث</v>
       </c>
       <c r="C118" t="str">
-        <v>Data Intelligence Center</v>
+        <v>Heritage Studio</v>
       </c>
       <c r="D118" t="str">
         <v/>
@@ -6558,10 +6558,10 @@
         <v>T118</v>
       </c>
       <c r="B119" t="str">
-        <v>أدوات إدارة وتحليل وتوثيق البيانات</v>
+        <v>أدوات إبداعية وعملية تنقل المنصة لمستوى آخر</v>
       </c>
       <c r="C119" t="str">
-        <v>Data management, analysis &amp; documentation tools</v>
+        <v>Creative &amp; practical tools that take the platform further</v>
       </c>
       <c r="D119" t="str">
         <v/>
@@ -6578,10 +6578,10 @@
         <v>T119</v>
       </c>
       <c r="B120" t="str">
-        <v>اكتشافات تلقائية</v>
+        <v>المتصفح لا يدعم تسجيل الفيديو</v>
       </c>
       <c r="C120" t="str">
-        <v>Auto insights</v>
+        <v>This browser does not support video recording</v>
       </c>
       <c r="D120" t="str">
         <v/>
@@ -6598,10 +6598,10 @@
         <v>T120</v>
       </c>
       <c r="B121" t="str">
-        <v>أنماط إحصائية مستخرجة آلياً من السجل الحالي (يتبع الفلاتر)</v>
+        <v>لا توجد قرى كافية</v>
       </c>
       <c r="C121" t="str">
-        <v>Statistical patterns mined from the currently filtered register</v>
+        <v>Not enough villages</v>
       </c>
       <c r="D121" t="str">
         <v/>
@@ -6618,10 +6618,10 @@
         <v>T121</v>
       </c>
       <c r="B122" t="str">
-        <v>لا توجد أنماط كافية ضمن الفلتر الحالي</v>
+        <v>تعذّر بدء التسجيل</v>
       </c>
       <c r="C122" t="str">
-        <v>Not enough data in the current filter</v>
+        <v>Could not start recording</v>
       </c>
       <c r="D122" t="str">
         <v/>
@@ -6638,10 +6638,10 @@
         <v>T122</v>
       </c>
       <c r="B123" t="str">
-        <v>هذه ملاحظات إحصائية آلية وليست استنتاجات نهائية — استخدمها كنقطة انطلاق للتحقق الميداني.</v>
+        <v>✓ تم حفظ الفيديو — شاهده أو شاركه مباشرة</v>
       </c>
       <c r="C123" t="str">
-        <v>Automated statistical observations, not final conclusions — use as a starting point for field verification.</v>
+        <v>✓ Video saved — watch or share it</v>
       </c>
       <c r="D123" t="str">
         <v/>
@@ -6658,10 +6658,10 @@
         <v>T123</v>
       </c>
       <c r="B124" t="str">
-        <v>فحص جودة البيانات</v>
+        <v>التسجيل كان قصيراً جداً</v>
       </c>
       <c r="C124" t="str">
-        <v>Data integrity scan</v>
+        <v>Recording too short</v>
       </c>
       <c r="D124" t="str">
         <v/>
@@ -6678,10 +6678,10 @@
         <v>T124</v>
       </c>
       <c r="B125" t="str">
-        <v>يفحص كامل السجل (٢٠,٨٠٠ موقع) عن مشاكل شائعة</v>
+        <v>تم إغلاق عدسة الزمن</v>
       </c>
       <c r="C125" t="str">
-        <v>Scans the full register for common issues</v>
+        <v>Time lens closed</v>
       </c>
       <c r="D125" t="str">
         <v/>
@@ -6698,10 +6698,10 @@
         <v>T125</v>
       </c>
       <c r="B126" t="str">
-        <v>جارِ الفحص…</v>
+        <v>🔮 اسحب العدسة فوق أي منطقة — داخلها ترى ٢٠٤٦</v>
       </c>
       <c r="C126" t="str">
-        <v>Scanning…</v>
+        <v>🔮 Drag the lens — inside it you see 2046</v>
       </c>
       <c r="D126" t="str">
         <v/>
@@ -6718,10 +6718,10 @@
         <v>T126</v>
       </c>
       <c r="B127" t="str">
-        <v>مجموعات إحداثيات متطابقة تقريباً</v>
+        <v>السجل الوطني مكتمل ✓</v>
       </c>
       <c r="C127" t="str">
-        <v>near-duplicate coordinate groups</v>
+        <v>National register complete ✓</v>
       </c>
       <c r="D127" t="str">
         <v/>
@@ -6738,10 +6738,10 @@
         <v>T127</v>
       </c>
       <c r="B128" t="str">
-        <v>إحداثيات خارج حدود المملكة تقريباً</v>
+        <v>محاكي «ماذا لو رمّمنا؟»</v>
       </c>
       <c r="C128" t="str">
-        <v>coords outside approx. KSA bounds</v>
+        <v>Restoration what-if simulator</v>
       </c>
       <c r="D128" t="str">
         <v/>
@@ -6758,10 +6758,10 @@
         <v>T128</v>
       </c>
       <c r="B129" t="str">
-        <v>قيم عمر/تهدّم غير منطقية</v>
+        <v>اختر نطاق ترميم افتراضي وشاهد أثره الفوري على مؤشر صحة التراث الوطني</v>
       </c>
       <c r="C129" t="str">
-        <v>implausible age/decay values</v>
+        <v>Pick a hypothetical restoration scope and watch the national index respond</v>
       </c>
       <c r="D129" t="str">
         <v/>
@@ -6778,10 +6778,10 @@
         <v>T129</v>
       </c>
       <c r="B130" t="str">
-        <v>عرض</v>
+        <v>أعلى ١٠٠ موقع خطورة</v>
       </c>
       <c r="C130" t="str">
-        <v>View</v>
+        <v>Top 100 risky</v>
       </c>
       <c r="D130" t="str">
         <v/>
@@ -6798,10 +6798,10 @@
         <v>T130</v>
       </c>
       <c r="B131" t="str">
-        <v>لا يوجد</v>
+        <v>كل الفلتر الحالي</v>
       </c>
       <c r="C131" t="str">
-        <v>None found</v>
+        <v>Entire current filter</v>
       </c>
       <c r="D131" t="str">
         <v/>
@@ -6818,10 +6818,10 @@
         <v>T131</v>
       </c>
       <c r="B132" t="str">
-        <v>تقدير تكلفة الترميم</v>
+        <v>منطقة كاملة:</v>
       </c>
       <c r="C132" t="str">
-        <v>Restoration cost estimate</v>
+        <v>Whole region:</v>
       </c>
       <c r="D132" t="str">
         <v/>
@@ -6838,10 +6838,10 @@
         <v>T132</v>
       </c>
       <c r="B133" t="str">
-        <v>تقدير تقريبي غير رسمي بناءً على نسبة التهدّم والفئة والنوع</v>
+        <v>أظهر الأثر على الخريطة ٥ ثوانٍ</v>
       </c>
       <c r="C133" t="str">
-        <v>Rough, unofficial estimate from decay %, class &amp; type</v>
+        <v>Show effect on map for 5s</v>
       </c>
       <c r="D133" t="str">
         <v/>
@@ -6858,10 +6858,10 @@
         <v>T133</v>
       </c>
       <c r="B134" t="str">
-        <v>مليار</v>
+        <v>الترميم الافتراضي = خفض تهدّم المواقع المختارة إلى ١٠٪. المؤشر الوطني يُحسب على كامل السجل.</v>
       </c>
       <c r="C134" t="str">
-        <v>B</v>
+        <v>Hypothetical restoration = selected sites decay drops to 10%. Index computed over the full register.</v>
       </c>
       <c r="D134" t="str">
         <v/>
@@ -6878,10 +6878,10 @@
         <v>T134</v>
       </c>
       <c r="B135" t="str">
-        <v>مليون</v>
+        <v>اليوم</v>
       </c>
       <c r="C135" t="str">
-        <v>M</v>
+        <v>Today</v>
       </c>
       <c r="D135" t="str">
         <v/>
@@ -6898,10 +6898,10 @@
         <v>T135</v>
       </c>
       <c r="B136" t="str">
-        <v>ر.س</v>
+        <v>نقطة</v>
       </c>
       <c r="C136" t="str">
-        <v>SAR</v>
+        <v>pts</v>
       </c>
       <c r="D136" t="str">
         <v/>
@@ -6918,10 +6918,10 @@
         <v>T136</v>
       </c>
       <c r="B137" t="str">
-        <v>إجمالي تقديري للمُصفّى الحالي</v>
+        <v>بعد الترميم</v>
       </c>
       <c r="C137" t="str">
-        <v>estimated total for current filter</v>
+        <v>After restoration</v>
       </c>
       <c r="D137" t="str">
         <v/>
@@ -6938,10 +6938,10 @@
         <v>T137</v>
       </c>
       <c r="B138" t="str">
-        <v>متوسط لكل موقع</v>
+        <v>موقع في خطة الترميم</v>
       </c>
       <c r="C138" t="str">
-        <v>avg per site</v>
+        <v>sites in the plan</v>
       </c>
       <c r="D138" t="str">
         <v/>
@@ -6958,10 +6958,10 @@
         <v>T138</v>
       </c>
       <c r="B139" t="str">
-        <v>أعلى ١٠ مناطق تكلفة تقديرية</v>
+        <v>مواقع تخرج من قائمة الملحّة</v>
       </c>
       <c r="C139" t="str">
-        <v>Top 10 regions by estimated cost</v>
+        <v>sites leave the urgent list</v>
       </c>
       <c r="D139" t="str">
         <v/>
@@ -6978,10 +6978,10 @@
         <v>T139</v>
       </c>
       <c r="B140" t="str">
-        <v>وضع الجدول الحي</v>
+        <v>المواقع الخضراء = خطة الترميم الافتراضية</v>
       </c>
       <c r="C140" t="str">
-        <v>Live spreadsheet</v>
+        <v>Green sites = the hypothetical plan</v>
       </c>
       <c r="D140" t="str">
         <v/>
@@ -6998,10 +6998,10 @@
         <v>T140</v>
       </c>
       <c r="B141" t="str">
-        <v>عدّل نسبة التهدّم، العمر، والفئة مباشرة — يُحفظ محلياً فوراً</v>
+        <v>قصص القرى التفاعلية</v>
       </c>
       <c r="C141" t="str">
-        <v>Edit decay, age &amp; class inline — saved locally instantly</v>
+        <v>Interactive village stories</v>
       </c>
       <c r="D141" t="str">
         <v/>
@@ -7018,10 +7018,10 @@
         <v>T141</v>
       </c>
       <c r="B142" t="str">
-        <v>الكود</v>
+        <v>اختر قرية — وستتحول لرحلة سردية فصولها مبانٍ حقيقية على الخريطة</v>
       </c>
       <c r="C142" t="str">
-        <v>Code</v>
+        <v>Pick a village — it becomes a guided narrative over the map</v>
       </c>
       <c r="D142" t="str">
         <v/>
@@ -7038,10 +7038,10 @@
         <v>T142</v>
       </c>
       <c r="B143" t="str">
-        <v>الاسم</v>
+        <v>الفصل</v>
       </c>
       <c r="C143" t="str">
-        <v>Name</v>
+        <v>Chapter</v>
       </c>
       <c r="D143" t="str">
         <v/>
@@ -7058,10 +7058,10 @@
         <v>T143</v>
       </c>
       <c r="B144" t="str">
-        <v>الفئة</v>
+        <v>مبنى تراثي موثّق</v>
       </c>
       <c r="C144" t="str">
-        <v>Class</v>
+        <v>documented heritage buildings</v>
       </c>
       <c r="D144" t="str">
         <v/>
@@ -7078,10 +7078,10 @@
         <v>T144</v>
       </c>
       <c r="B145" t="str">
-        <v>العمر</v>
+        <v>مرّر بالعجلة أو الأسهم لبدء الرحلة ↓</v>
       </c>
       <c r="C145" t="str">
-        <v>Age</v>
+        <v>Scroll or use arrows to begin ↓</v>
       </c>
       <c r="D145" t="str">
         <v/>
@@ -7098,10 +7098,10 @@
         <v>T145</v>
       </c>
       <c r="B146" t="str">
-        <v>التهدّم %</v>
+        <v>الفئة</v>
       </c>
       <c r="C146" t="str">
-        <v>Decay %</v>
+        <v>Class</v>
       </c>
       <c r="D146" t="str">
         <v/>
@@ -7118,10 +7118,10 @@
         <v>T146</v>
       </c>
       <c r="B147" t="str">
-        <v>السابق</v>
+        <v>التهدّم</v>
       </c>
       <c r="C147" t="str">
-        <v>Prev</v>
+        <v>Decay</v>
       </c>
       <c r="D147" t="str">
         <v/>
@@ -7138,10 +7138,10 @@
         <v>T147</v>
       </c>
       <c r="B148" t="str">
-        <v>التالي</v>
+        <v>العمر</v>
       </c>
       <c r="C148" t="str">
-        <v>Next</v>
+        <v>Age</v>
       </c>
       <c r="D148" t="str">
         <v/>
@@ -7158,10 +7158,10 @@
         <v>T148</v>
       </c>
       <c r="B149" t="str">
-        <v>تم الحفظ</v>
+        <v>مواد البناء</v>
       </c>
       <c r="C149" t="str">
-        <v>Saved</v>
+        <v>Materials</v>
       </c>
       <c r="D149" t="str">
         <v/>
@@ -7178,10 +7178,10 @@
         <v>T149</v>
       </c>
       <c r="B150" t="str">
-        <v>استيراد ذكي</v>
+        <v>التفاصيل الكاملة</v>
       </c>
       <c r="C150" t="str">
-        <v>Smart importer</v>
+        <v>Full details</v>
       </c>
       <c r="D150" t="str">
         <v/>
@@ -7198,10 +7198,10 @@
         <v>T150</v>
       </c>
       <c r="B151" t="str">
-        <v>ارفع ملف CSV — سيتم التعرف على الأعمدة تلقائياً ودمج المواقع الجديدة</v>
+        <v>🗺️ وضع المخطوطة العتيقة مفعّل</v>
       </c>
       <c r="C151" t="str">
-        <v>Upload a CSV — columns are auto-detected and new sites merged</v>
+        <v>🗺️ Vintage manuscript mode on</v>
       </c>
       <c r="D151" t="str">
         <v/>
@@ -7218,10 +7218,10 @@
         <v>T151</v>
       </c>
       <c r="B152" t="str">
-        <v>اسحب ملف CSV هنا أو اضغط للاختيار</v>
+        <v>عدنا للخريطة الحديثة</v>
       </c>
       <c r="C152" t="str">
-        <v>Drag a CSV file here or click to choose</v>
+        <v>Back to the modern map</v>
       </c>
       <c r="D152" t="str">
         <v/>
@@ -7238,10 +7238,10 @@
         <v>T152</v>
       </c>
       <c r="B153" t="str">
-        <v>يدعم الأعمدة: الاسم، خط العرض، خط الطول، المنطقة، المحافظة، العمر، التهدّم، الفئة</v>
+        <v>مولّد اللوحات التعريفية الميدانية</v>
       </c>
       <c r="C153" t="str">
-        <v>Supports: name, lat, lng, region, governorate, age, decay, class</v>
+        <v>Field plaque generator</v>
       </c>
       <c r="D153" t="str">
         <v/>
@@ -7258,10 +7258,10 @@
         <v>T153</v>
       </c>
       <c r="B154" t="str">
-        <v>الملف فارغ أو غير صالح</v>
+        <v>لوحات A5 وملصقات QR جاهزة للطباعة والتثبيت على المواقع نفسها</v>
       </c>
       <c r="C154" t="str">
-        <v>Empty or invalid file</v>
+        <v>Print-ready A5 plaques &amp; QR sticker sheets for the physical sites</v>
       </c>
       <c r="D154" t="str">
         <v/>
@@ -7278,10 +7278,10 @@
         <v>T154</v>
       </c>
       <c r="B155" t="str">
-        <v>تعذّر التعرف على أعمدة الاسم/الإحداثيات. تأكد من وجود أعمدة باسم أو Name وLat/Lng.</v>
+        <v>عدد المواقع (الأعلى خطورة من الفلتر الحالي)</v>
       </c>
       <c r="C155" t="str">
-        <v>Could not detect name/coordinate columns. Make sure Name and Lat/Lng columns exist.</v>
+        <v>Site count (top risky from current filter)</v>
       </c>
       <c r="D155" t="str">
         <v/>
@@ -7298,10 +7298,10 @@
         <v>T155</v>
       </c>
       <c r="B156" t="str">
-        <v>صف صالح</v>
+        <v>لوحات A5 (لوحة لكل موقع)</v>
       </c>
       <c r="C156" t="str">
-        <v>valid rows</v>
+        <v>A5 plaques (one per site)</v>
       </c>
       <c r="D156" t="str">
         <v/>
@@ -7318,10 +7318,10 @@
         <v>T156</v>
       </c>
       <c r="B157" t="str">
-        <v>يبدو مكرراً (سيُتجاهل)</v>
+        <v>ملصقات QR (8 لكل صفحة)</v>
       </c>
       <c r="C157" t="str">
-        <v>looks duplicate (will be skipped)</v>
+        <v>QR stickers (8 per page)</v>
       </c>
       <c r="D157" t="str">
         <v/>
@@ -7338,10 +7338,10 @@
         <v>T157</v>
       </c>
       <c r="B158" t="str">
-        <v>مكرر محتمل</v>
+        <v>كل لوحة تحمل اسم الموقع وفئته ورمز QR يفتح صفحته الكاملة على المنصة — ثبّتها على المبنى ليصبح متصلاً بسجله الرقمي.</v>
       </c>
       <c r="C158" t="str">
-        <v>possible dup</v>
+        <v>Each plaque carries the site name, class and a QR opening its full page — mount it on the building to link it to its digital record.</v>
       </c>
       <c r="D158" t="str">
         <v/>
@@ -7358,10 +7358,10 @@
         <v>T158</v>
       </c>
       <c r="B159" t="str">
-        <v>تعذّر قراءة الملف</v>
+        <v>امسح الرمز لفتح السجل الرقمي الكامل لهذا الأصل</v>
       </c>
       <c r="C159" t="str">
-        <v>Could not read file</v>
+        <v>Scan to open this asset’s full digital record</v>
       </c>
       <c r="D159" t="str">
         <v/>
@@ -7378,10 +7378,10 @@
         <v>T159</v>
       </c>
       <c r="B160" t="str">
-        <v>موقع مستورد</v>
+        <v>الخريطة الحرارية عبر الزمن</v>
       </c>
       <c r="C160" t="str">
-        <v>sites imported</v>
+        <v>Temporal heat map</v>
       </c>
       <c r="D160" t="str">
         <v/>
@@ -7398,10 +7398,10 @@
         <v>T160</v>
       </c>
       <c r="B161" t="str">
-        <v>آلة الزمن</v>
+        <v>شاهد كثافة التراث تتشكل من الأقدم إلى الأحدث</v>
       </c>
       <c r="C161" t="str">
-        <v>Time machine</v>
+        <v>Watch heritage density bloom from oldest to newest</v>
       </c>
       <c r="D161" t="str">
         <v/>
@@ -7418,10 +7418,10 @@
         <v>T161</v>
       </c>
       <c r="B162" t="str">
-        <v>لقطات مؤشرات محفوظة محلياً لمقارنة تطوّر السجل عبر الزمن</v>
+        <v>تشغيل الرحلة</v>
       </c>
       <c r="C162" t="str">
-        <v>Locally saved KPI snapshots to compare register growth over time</v>
+        <v>Play the journey</v>
       </c>
       <c r="D162" t="str">
         <v/>
@@ -7438,10 +7438,10 @@
         <v>T162</v>
       </c>
       <c r="B163" t="str">
-        <v>موقع</v>
+        <v>موقع ظاهر في الطبقة الحرارية</v>
       </c>
       <c r="C163" t="str">
-        <v>sites</v>
+        <v>sites in the heat layer</v>
       </c>
       <c r="D163" t="str">
         <v/>
@@ -7458,10 +7458,10 @@
         <v>T163</v>
       </c>
       <c r="B164" t="str">
-        <v>ملحّة</v>
+        <v>اسحب: يمين = مواقع أقدم فقط. الطبقة الحرارية مفعّلة تلقائياً أثناء العرض.</v>
       </c>
       <c r="C164" t="str">
-        <v>urgent</v>
+        <v>Drag right = only older sites. Heat layer auto-enabled while open.</v>
       </c>
       <c r="D164" t="str">
         <v/>
@@ -7478,10 +7478,10 @@
         <v>T164</v>
       </c>
       <c r="B165" t="str">
-        <v>الحالي</v>
+        <v>موقع</v>
       </c>
       <c r="C165" t="str">
-        <v>current total</v>
+        <v>sites</v>
       </c>
       <c r="D165" t="str">
         <v/>
@@ -7498,10 +7498,10 @@
         <v>T165</v>
       </c>
       <c r="B166" t="str">
-        <v>متوسط التهدّم الآن</v>
+        <v>الاستيراد الذكي</v>
       </c>
       <c r="C166" t="str">
-        <v>current avg decay</v>
+        <v>Smart importer</v>
       </c>
       <c r="D166" t="str">
         <v/>
@@ -7518,10 +7518,10 @@
         <v>T166</v>
       </c>
       <c r="B167" t="str">
-        <v>حفظ لقطة الآن</v>
+        <v>ارفع ملف CSV — سيتم التعرف على الأعمدة تلقائياً ودمج المواقع الجديدة</v>
       </c>
       <c r="C167" t="str">
-        <v>Save snapshot now</v>
+        <v>Upload a CSV — columns are auto-detected and new sites merged</v>
       </c>
       <c r="D167" t="str">
         <v/>
@@ -7538,10 +7538,10 @@
         <v>T167</v>
       </c>
       <c r="B168" t="str">
-        <v>اللقطات المحفوظة</v>
+        <v>اسحب ملف CSV هنا أو اضغط للاختيار</v>
       </c>
       <c r="C168" t="str">
-        <v>Saved snapshots</v>
+        <v>Drag a CSV file here or click to choose</v>
       </c>
       <c r="D168" t="str">
         <v/>
@@ -7558,10 +7558,10 @@
         <v>T168</v>
       </c>
       <c r="B169" t="str">
-        <v>لا لقطات بعد</v>
+        <v>يدعم الأعمدة: الاسم، خط العرض، خط الطول، المنطقة، المحافظة، العمر، التهدّم، الفئة</v>
       </c>
       <c r="C169" t="str">
-        <v>No snapshots yet</v>
+        <v>Supports: name, lat, lng, region, governorate, age, decay, class</v>
       </c>
       <c r="D169" t="str">
         <v/>
@@ -7578,10 +7578,10 @@
         <v>T169</v>
       </c>
       <c r="B170" t="str">
-        <v>✓ تم حفظ اللقطة</v>
+        <v>الملف فارغ أو غير صالح</v>
       </c>
       <c r="C170" t="str">
-        <v>✓ Snapshot saved</v>
+        <v>Empty or invalid file</v>
       </c>
       <c r="D170" t="str">
         <v/>
@@ -7598,10 +7598,10 @@
         <v>T170</v>
       </c>
       <c r="B171" t="str">
-        <v>حماية التعديل</v>
+        <v>تعذّر التعرف على أعمدة الاسم/الإحداثيات. تأكد من وجود أعمدة باسم أو Name وLat/Lng.</v>
       </c>
       <c r="C171" t="str">
-        <v>Edit protection</v>
+        <v>Could not detect name/coordinate columns. Make sure Name and Lat/Lng columns exist.</v>
       </c>
       <c r="D171" t="str">
         <v/>
@@ -7618,10 +7618,10 @@
         <v>T171</v>
       </c>
       <c r="B172" t="str">
-        <v>قفل محلي بسيط لمنع التعديل العرضي على هذا الجهاز — ليس تشفيراً أمنياً</v>
+        <v>صف صالح</v>
       </c>
       <c r="C172" t="str">
-        <v>A simple local guard against accidental edits on this device — not real security</v>
+        <v>valid rows</v>
       </c>
       <c r="D172" t="str">
         <v/>
@@ -7638,10 +7638,10 @@
         <v>T172</v>
       </c>
       <c r="B173" t="str">
-        <v>التعديل مقفل حالياً على هذا الجهاز.</v>
+        <v>يبدو مكرراً (سيُتجاهل)</v>
       </c>
       <c r="C173" t="str">
-        <v>Editing is currently locked on this device.</v>
+        <v>looks duplicate (will be skipped)</v>
       </c>
       <c r="D173" t="str">
         <v/>
@@ -7658,10 +7658,10 @@
         <v>T173</v>
       </c>
       <c r="B174" t="str">
-        <v>كلمة المرور</v>
+        <v>مكرر محتمل</v>
       </c>
       <c r="C174" t="str">
-        <v>Passphrase</v>
+        <v>possible dup</v>
       </c>
       <c r="D174" t="str">
         <v/>
@@ -7678,10 +7678,10 @@
         <v>T174</v>
       </c>
       <c r="B175" t="str">
-        <v>فتح القفل</v>
+        <v>تعذّر قراءة الملف</v>
       </c>
       <c r="C175" t="str">
-        <v>Unlock</v>
+        <v>Could not read file</v>
       </c>
       <c r="D175" t="str">
         <v/>
@@ -7698,10 +7698,10 @@
         <v>T175</v>
       </c>
       <c r="B176" t="str">
-        <v>✓ تم فتح القفل</v>
+        <v>موقع مستورد</v>
       </c>
       <c r="C176" t="str">
-        <v>✓ Unlocked</v>
+        <v>sites imported</v>
       </c>
       <c r="D176" t="str">
         <v/>
@@ -7718,10 +7718,10 @@
         <v>T176</v>
       </c>
       <c r="B177" t="str">
-        <v>كلمة مرور خاطئة</v>
+        <v>آلة الزمن</v>
       </c>
       <c r="C177" t="str">
-        <v>Wrong passphrase</v>
+        <v>Time machine</v>
       </c>
       <c r="D177" t="str">
         <v/>
@@ -7738,10 +7738,10 @@
         <v>T177</v>
       </c>
       <c r="B178" t="str">
-        <v>عند التفعيل، ستحتاج لإدخال كلمة المرور قبل إضافة مواقع أو استيراد بيانات على هذا الجهاز.</v>
+        <v>لقطات مؤشرات محفوظة محلياً لمقارنة تطوّر السجل عبر الزمن</v>
       </c>
       <c r="C178" t="str">
-        <v>Once enabled, you will need the passphrase before adding sites or importing data on this device.</v>
+        <v>Locally saved KPI snapshots to compare register growth over time</v>
       </c>
       <c r="D178" t="str">
         <v/>
@@ -7758,10 +7758,10 @@
         <v>T178</v>
       </c>
       <c r="B179" t="str">
-        <v>اختر كلمة مرور</v>
+        <v>ملحّة</v>
       </c>
       <c r="C179" t="str">
-        <v>Choose a passphrase</v>
+        <v>urgent</v>
       </c>
       <c r="D179" t="str">
         <v/>
@@ -7778,10 +7778,10 @@
         <v>T179</v>
       </c>
       <c r="B180" t="str">
-        <v>تفعيل القفل</v>
+        <v>الحالي</v>
       </c>
       <c r="C180" t="str">
-        <v>Enable lock</v>
+        <v>current total</v>
       </c>
       <c r="D180" t="str">
         <v/>
@@ -7798,10 +7798,10 @@
         <v>T180</v>
       </c>
       <c r="B181" t="str">
-        <v>اكتب ٣ أحرف على الأقل</v>
+        <v>متوسط التهدّم الآن</v>
       </c>
       <c r="C181" t="str">
-        <v>Use at least 3 characters</v>
+        <v>current avg decay</v>
       </c>
       <c r="D181" t="str">
         <v/>
@@ -7818,10 +7818,10 @@
         <v>T181</v>
       </c>
       <c r="B182" t="str">
-        <v>✓ تم تفعيل القفل</v>
+        <v>حفظ لقطة الآن</v>
       </c>
       <c r="C182" t="str">
-        <v>✓ Lock enabled</v>
+        <v>Save snapshot now</v>
       </c>
       <c r="D182" t="str">
         <v/>
@@ -7838,10 +7838,10 @@
         <v>T182</v>
       </c>
       <c r="B183" t="str">
-        <v>أدخل كلمة مرور التعديل:</v>
+        <v>اللقطات المحفوظة</v>
       </c>
       <c r="C183" t="str">
-        <v>Enter the edit passphrase:</v>
+        <v>Saved snapshots</v>
       </c>
       <c r="D183" t="str">
         <v/>
@@ -7858,10 +7858,10 @@
         <v>T183</v>
       </c>
       <c r="B184" t="str">
-        <v>عرض كـ JSON</v>
+        <v>لا لقطات بعد</v>
       </c>
       <c r="C184" t="str">
-        <v>View as JSON</v>
+        <v>No snapshots yet</v>
       </c>
       <c r="D184" t="str">
         <v/>
@@ -7878,10 +7878,10 @@
         <v>T184</v>
       </c>
       <c r="B185" t="str">
-        <v>نسخة من البيانات المُصفّاة الحالية بصيغة JSON منظمة — للاستخدام في أنظمة أو أدوات أخرى</v>
+        <v>✓ تم حفظ اللقطة</v>
       </c>
       <c r="C185" t="str">
-        <v>A shaped JSON snapshot of the current filter — for other systems/tools</v>
+        <v>✓ Snapshot saved</v>
       </c>
       <c r="D185" t="str">
         <v/>
@@ -7898,10 +7898,10 @@
         <v>T185</v>
       </c>
       <c r="B186" t="str">
-        <v>موقع في هذه اللقطة</v>
+        <v>الاستوديو</v>
       </c>
       <c r="C186" t="str">
-        <v>sites in this snapshot</v>
+        <v>Studio</v>
       </c>
       <c r="D186" t="str">
         <v/>
@@ -7918,10 +7918,10 @@
         <v>T186</v>
       </c>
       <c r="B187" t="str">
-        <v>مقتطف — نزّل الملف للنسخة الكاملة</v>
+        <v>جارِ تسجيل الجولة</v>
       </c>
       <c r="C187" t="str">
-        <v>truncated — download for full file</v>
+        <v>Recording tour</v>
       </c>
       <c r="D187" t="str">
         <v/>
@@ -7938,10 +7938,10 @@
         <v>T187</v>
       </c>
       <c r="B188" t="str">
-        <v>تنزيل JSON</v>
+        <v>إيقاف وحفظ</v>
       </c>
       <c r="C188" t="str">
-        <v>Download JSON</v>
+        <v>Stop &amp; save</v>
       </c>
       <c r="D188" t="str">
         <v/>
@@ -7958,10 +7958,10 @@
         <v>T188</v>
       </c>
       <c r="B189" t="str">
-        <v>نسخ</v>
+        <v>أصل تراثي موثّق</v>
       </c>
       <c r="C189" t="str">
-        <v>Copy</v>
+        <v>heritage assets documented</v>
       </c>
       <c r="D189" t="str">
         <v/>
@@ -7978,10 +7978,10 @@
         <v>T189</v>
       </c>
       <c r="B190" t="str">
-        <v>تم النسخ</v>
+        <v>السابق</v>
       </c>
       <c r="C190" t="str">
-        <v>Copied</v>
+        <v>Previous</v>
       </c>
       <c r="D190" t="str">
         <v/>
@@ -7998,10 +7998,10 @@
         <v>T190</v>
       </c>
       <c r="B191" t="str">
-        <v>مؤشّر المخاطر البيئية التقديري</v>
+        <v>التالي</v>
       </c>
       <c r="C191" t="str">
-        <v>Estimated environmental risk</v>
+        <v>Next</v>
       </c>
       <c r="D191" t="str">
         <v/>
@@ -8018,10 +8018,10 @@
         <v>T191</v>
       </c>
       <c r="B192" t="str">
-        <v>تقدير تقريبي من الارتفاع والموقع الجغرافي (بدون اتصال بخدمات خارجية) — وليس بيانات رصد جوي حقيقية</v>
+        <v>إنهاء القصة</v>
       </c>
       <c r="C192" t="str">
-        <v>Approximate estimate from elevation &amp; location (fully offline) — not real weather data</v>
+        <v>End story</v>
       </c>
       <c r="D192" t="str">
         <v/>
@@ -8038,10 +8038,10 @@
         <v>T192</v>
       </c>
       <c r="B193" t="str">
-        <v>متوسط المؤشر (٠-١٠٠)</v>
+        <v>مقارنة منطقتين — خريطتان متزامنتان</v>
       </c>
       <c r="C193" t="str">
-        <v>avg index (0-100)</v>
+        <v>Two regions — synced maps</v>
       </c>
       <c r="D193" t="str">
         <v/>
@@ -8058,10 +8058,10 @@
         <v>T193</v>
       </c>
       <c r="B194" t="str">
-        <v>الأعلى عرضة تقديرياً</v>
+        <v>لم أجد أي موقع مطابق (${scope}).</v>
       </c>
       <c r="C194" t="str">
-        <v>Highest estimated exposure</v>
+        <v>No sites matched (${scope}).</v>
       </c>
       <c r="D194" t="str">
         <v/>
@@ -8070,7 +8070,7 @@
         <v/>
       </c>
       <c r="F194" t="str">
-        <v/>
+        <v>ديناميكي — لا تلمس ${...}</v>
       </c>
     </row>
     <row r="195">
@@ -8078,10 +8078,10 @@
         <v>T194</v>
       </c>
       <c r="B195" t="str">
-        <v>موسوعة الطرز المعمارية</v>
+        <v>أعلى ${num(top.length)} مواقع خطورة (${scope}) — اضغط أي موقع للانتقال إليه:</v>
       </c>
       <c r="C195" t="str">
-        <v>Architectural style encyclopedia</v>
+        <v>Top ${num(top.length)} risky sites (${scope}):</v>
       </c>
       <c r="D195" t="str">
         <v/>
@@ -8090,7 +8090,7 @@
         <v/>
       </c>
       <c r="F195" t="str">
-        <v/>
+        <v>ديناميكي — لا تلمس ${...}</v>
       </c>
     </row>
     <row r="196">
@@ -8098,10 +8098,10 @@
         <v>T195</v>
       </c>
       <c r="B196" t="str">
-        <v>الطرز المسجّلة في السجل الحالي مع عدد المواقع</v>
+        <v>أعلى ${num(Math.min(100,top.length))} موقعاً حسب مؤشّر المخاطر المركّب (تهدّم × أهمية × غياب أعمال)</v>
       </c>
       <c r="C196" t="str">
-        <v>Styles present in the register, with site counts</v>
+        <v>Top ${num(Math.min(100,top.length))} by composite risk</v>
       </c>
       <c r="D196" t="str">
         <v/>
@@ -8110,7 +8110,7 @@
         <v/>
       </c>
       <c r="F196" t="str">
-        <v/>
+        <v>ديناميكي — لا تلمس ${...}</v>
       </c>
     </row>
     <row r="197">
@@ -8118,10 +8118,10 @@
         <v>T196</v>
       </c>
       <c r="B197" t="str">
-        <v>لا بيانات طراز مسجّلة</v>
+        <v>اعرض المواقع التي يبلغ عمرها كذا سنة فأكثر (${num(withAge)} موقعاً له عمر مسجّل)</v>
       </c>
       <c r="C197" t="str">
-        <v>No style data recorded</v>
+        <v>Show sites at least N years old (${num(withAge)} dated)</v>
       </c>
       <c r="D197" t="str">
         <v/>
@@ -8130,7 +8130,7 @@
         <v/>
       </c>
       <c r="F197" t="str">
-        <v/>
+        <v>ديناميكي — لا تلمس ${...}</v>
       </c>
     </row>
     <row r="198">
@@ -8138,10 +8138,10 @@
         <v>T197</v>
       </c>
       <c r="B198" t="str">
-        <v>اضغط أي طراز لعرض مواقعه على الخريطة.</v>
+        <v>${num(vs.length)} قرية تراثية مكتشفة تلقائياً من أسماء المواقع</v>
       </c>
       <c r="C198" t="str">
-        <v>Click a style to view its sites on the map.</v>
+        <v>${num(vs.length)} villages auto-detected</v>
       </c>
       <c r="D198" t="str">
         <v/>
@@ -8150,7 +8150,7 @@
         <v/>
       </c>
       <c r="F198" t="str">
-        <v/>
+        <v>ديناميكي — لا تلمس ${...}</v>
       </c>
     </row>
     <row r="199">
@@ -8158,10 +8158,10 @@
         <v>T198</v>
       </c>
       <c r="B199" t="str">
-        <v>العصور التاريخية (تقديرية)</v>
+        <v>نطاقات حماية ٥٠٠م حول ${num(pts.length)} موقع فئة (أ) — كبّر الخريطة لرؤيتها</v>
       </c>
       <c r="C199" t="str">
-        <v>Historical eras (approximate)</v>
+        <v>500m buffers on ${num(pts.length)} Class A sites — zoom in</v>
       </c>
       <c r="D199" t="str">
         <v/>
@@ -8170,7 +8170,7 @@
         <v/>
       </c>
       <c r="F199" t="str">
-        <v/>
+        <v>ديناميكي — لا تلمس ${...}</v>
       </c>
     </row>
     <row r="200">
@@ -8178,10 +8178,10 @@
         <v>T199</v>
       </c>
       <c r="B200" t="str">
-        <v>تصنيف حسب العمر التقريبي المسجّل — وليس تأريخاً أثرياً معتمداً</v>
+        <v>+ ${num(parsed.length-12)} صف آخر</v>
       </c>
       <c r="C200" t="str">
-        <v>Grouped by recorded approximate age — not a certified archaeological dating</v>
+        <v>+ ${num(parsed.length-12)} more rows</v>
       </c>
       <c r="D200" t="str">
         <v/>
@@ -8190,7 +8190,7 @@
         <v/>
       </c>
       <c r="F200" t="str">
-        <v/>
+        <v>ديناميكي — لا تلمس ${...}</v>
       </c>
     </row>
     <row r="201">
@@ -8198,10 +8198,10 @@
         <v>T200</v>
       </c>
       <c r="B201" t="str">
-        <v>لوحة القيادة التنفيذية</v>
+        <v>استيراد ${num(parsed.length-dupCount)} موقع</v>
       </c>
       <c r="C201" t="str">
-        <v>Executive Overview</v>
+        <v>Import ${num(parsed.length-dupCount)} sites</v>
       </c>
       <c r="D201" t="str">
         <v/>
@@ -8210,7 +8210,7 @@
         <v/>
       </c>
       <c r="F201" t="str">
-        <v/>
+        <v>ديناميكي — لا تلمس ${...}</v>
       </c>
     </row>
     <row r="202">
@@ -8218,10 +8218,10 @@
         <v>T201</v>
       </c>
       <c r="B202" t="str">
-        <v>متوسط التهدّم</v>
+        <v>✓ تم استيراد ${num(added)} موقع بنجاح</v>
       </c>
       <c r="C202" t="str">
-        <v>Avg deterioration</v>
+        <v>✓ Imported ${num(added)} sites successfully</v>
       </c>
       <c r="D202" t="str">
         <v/>
@@ -8230,7 +8230,7 @@
         <v/>
       </c>
       <c r="F202" t="str">
-        <v/>
+        <v>ديناميكي — لا تلمس ${...}</v>
       </c>
     </row>
     <row r="203">
@@ -8238,10 +8238,10 @@
         <v>T202</v>
       </c>
       <c r="B203" t="str">
-        <v>ملحّة للترميم</v>
+        <v>اضغط للتصفية على هذه المنطقة</v>
       </c>
       <c r="C203" t="str">
-        <v>Urgent restoration</v>
+        <v>Click to filter by this region</v>
       </c>
       <c r="D203" t="str">
         <v/>
@@ -8258,10 +8258,10 @@
         <v>T203</v>
       </c>
       <c r="B204" t="str">
-        <v>مناطق مشمولة</v>
+        <v>لوحة التحليلات</v>
       </c>
       <c r="C204" t="str">
-        <v>Regions covered</v>
+        <v>Analytics Dashboard</v>
       </c>
       <c r="D204" t="str">
         <v/>
@@ -8278,10 +8278,10 @@
         <v>T204</v>
       </c>
       <c r="B205" t="str">
-        <v>أعلى ٣ مواقع أولوية</v>
+        <v>تحليل شامل للأصول التراثية المعروضة حالياً</v>
       </c>
       <c r="C205" t="str">
-        <v>Top 3 priority sites</v>
+        <v>Comprehensive analysis of currently displayed heritage assets</v>
       </c>
       <c r="D205" t="str">
         <v/>
@@ -8298,10 +8298,10 @@
         <v>T205</v>
       </c>
       <c r="B206" t="str">
-        <v>مؤشّر مخاطر</v>
+        <v>متوسط نسبة التهدّم</v>
       </c>
       <c r="C206" t="str">
-        <v>risk index</v>
+        <v>Average deterioration</v>
       </c>
       <c r="D206" t="str">
         <v/>
@@ -8318,10 +8318,10 @@
         <v>T206</v>
       </c>
       <c r="B207" t="str">
-        <v>لا توجد مواقع ضمن الفلتر الحالي</v>
+        <v>مواقع ملحّة للترميم</v>
       </c>
       <c r="C207" t="str">
-        <v>No sites in current filter</v>
+        <v>Urgent for restoration</v>
       </c>
       <c r="D207" t="str">
         <v/>
@@ -8338,10 +8338,10 @@
         <v>T207</v>
       </c>
       <c r="B208" t="str">
-        <v>عرض تقديمي</v>
+        <v>متوسط العمر (سنة)</v>
       </c>
       <c r="C208" t="str">
-        <v>Presentation</v>
+        <v>Average age (yrs)</v>
       </c>
       <c r="D208" t="str">
         <v/>
@@ -8358,10 +8358,10 @@
         <v>T208</v>
       </c>
       <c r="B209" t="str">
-        <v>نظرة عامة</v>
+        <v>مناطق / محافظات</v>
       </c>
       <c r="C209" t="str">
-        <v>Overview</v>
+        <v>Regions / governorates</v>
       </c>
       <c r="D209" t="str">
         <v/>
@@ -8378,10 +8378,10 @@
         <v>T209</v>
       </c>
       <c r="B210" t="str">
-        <v>إجمالي</v>
+        <v>التوزيع حسب المنطقة</v>
       </c>
       <c r="C210" t="str">
-        <v>Total</v>
+        <v>Distribution by region</v>
       </c>
       <c r="D210" t="str">
         <v/>
@@ -8398,10 +8398,10 @@
         <v>T210</v>
       </c>
       <c r="B211" t="str">
-        <v>مناطق</v>
+        <v>فئة الأهمية</v>
       </c>
       <c r="C211" t="str">
-        <v>Regions</v>
+        <v>Significance class</v>
       </c>
       <c r="D211" t="str">
         <v/>
@@ -8418,10 +8418,10 @@
         <v>T211</v>
       </c>
       <c r="B212" t="str">
-        <v>ملحّة</v>
+        <v>مبنى</v>
       </c>
       <c r="C212" t="str">
-        <v>Urgent</v>
+        <v>buildings</v>
       </c>
       <c r="D212" t="str">
         <v/>
@@ -8438,10 +8438,10 @@
         <v>T212</v>
       </c>
       <c r="B213" t="str">
-        <v>موقع</v>
+        <v>منطقة</v>
       </c>
       <c r="C213" t="str">
-        <v>Site</v>
+        <v>zones</v>
       </c>
       <c r="D213" t="str">
         <v/>
@@ -8458,10 +8458,10 @@
         <v>T213</v>
       </c>
       <c r="B214" t="str">
-        <v>مؤشّر المخاطر</v>
+        <v>أعلى ١٠ محافظات</v>
       </c>
       <c r="C214" t="str">
-        <v>Risk index</v>
+        <v>Top 10 governorates</v>
       </c>
       <c r="D214" t="str">
         <v/>
@@ -8478,10 +8478,10 @@
         <v>T214</v>
       </c>
       <c r="B215" t="str">
-        <v>شكراً</v>
+        <v>نوع التراث</v>
       </c>
       <c r="C215" t="str">
-        <v>Thank you</v>
+        <v>Heritage type</v>
       </c>
       <c r="D215" t="str">
         <v/>
@@ -8498,10 +8498,10 @@
         <v>T215</v>
       </c>
       <c r="B216" t="str">
-        <v>يرجى السماح بالنوافذ المنبثقة</v>
+        <v>مؤشّر اكتمال البيانات</v>
       </c>
       <c r="C216" t="str">
-        <v>Please allow pop-ups</v>
+        <v>Data completeness</v>
       </c>
       <c r="D216" t="str">
         <v/>
@@ -8518,10 +8518,10 @@
         <v>T216</v>
       </c>
       <c r="B217" t="str">
-        <v>أطلس المحافظات</v>
+        <v>نسبة التهدّم</v>
       </c>
       <c r="C217" t="str">
-        <v>Governorate atlas</v>
+        <v>Deterioration %</v>
       </c>
       <c r="D217" t="str">
         <v/>
@@ -8538,10 +8538,10 @@
         <v>T217</v>
       </c>
       <c r="B218" t="str">
-        <v>اختر محافظة لطباعة تقرير مخصص لها</v>
+        <v>العمر التقريبي</v>
       </c>
       <c r="C218" t="str">
-        <v>Pick a governorate to print a dedicated report</v>
+        <v>Approx. age</v>
       </c>
       <c r="D218" t="str">
         <v/>
@@ -8558,10 +8558,10 @@
         <v>T218</v>
       </c>
       <c r="B219" t="str">
-        <v>تقرير محافظة</v>
+        <v>رقم القرار</v>
       </c>
       <c r="C219" t="str">
-        <v>Governorate Profile</v>
+        <v>Decision no.</v>
       </c>
       <c r="D219" t="str">
         <v/>
@@ -8578,10 +8578,10 @@
         <v>T219</v>
       </c>
       <c r="B220" t="str">
-        <v>المواقع المهملة</v>
+        <v>بيانات الحصر الميداني</v>
       </c>
       <c r="C220" t="str">
-        <v>Neglected sites</v>
+        <v>Field survey data</v>
       </c>
       <c r="D220" t="str">
         <v/>
@@ -8598,10 +8598,10 @@
         <v>T220</v>
       </c>
       <c r="B221" t="str">
-        <v>الأقل اكتمالاً في البيانات وبدون توثيق أو تعديل مسجّل مؤخراً</v>
+        <v>لا توجد نتائج</v>
       </c>
       <c r="C221" t="str">
-        <v>Least complete data, with no recently recorded documentation</v>
+        <v>No results</v>
       </c>
       <c r="D221" t="str">
         <v/>
@@ -8618,10 +8618,10 @@
         <v>T221</v>
       </c>
       <c r="B222" t="str">
-        <v>موقع بحاجة لمتابعة</v>
+        <v>عرض المزيد</v>
       </c>
       <c r="C222" t="str">
-        <v>sites needing follow-up</v>
+        <v>Show more</v>
       </c>
       <c r="D222" t="str">
         <v/>
@@ -8638,10 +8638,10 @@
         <v>T222</v>
       </c>
       <c r="B223" t="str">
-        <v>حقول ناقصة</v>
+        <v>نهاية القائمة</v>
       </c>
       <c r="C223" t="str">
-        <v>missing fields</v>
+        <v>End of list</v>
       </c>
       <c r="D223" t="str">
         <v/>
@@ -8658,10 +8658,10 @@
         <v>T223</v>
       </c>
       <c r="B224" t="str">
-        <v>السجل مكتمل جيداً ضمن الفلتر الحالي</v>
+        <v>أصل</v>
       </c>
       <c r="C224" t="str">
-        <v>Data looks well-completed for the current filter</v>
+        <v>assets</v>
       </c>
       <c r="D224" t="str">
         <v/>
@@ -8678,10 +8678,10 @@
         <v>T224</v>
       </c>
       <c r="B225" t="str">
-        <v>صور تاريخية عبر الأقمار الصناعية</v>
+        <v>لا توجد نتائج مطابقة</v>
       </c>
       <c r="C225" t="str">
-        <v>Historical satellite imagery</v>
+        <v>No matching results</v>
       </c>
       <c r="D225" t="str">
         <v/>
@@ -8698,10 +8698,10 @@
         <v>T225</v>
       </c>
       <c r="B226" t="str">
-        <v>يفتح أرشيف الصور التاريخية لموقع محدد في نافذة خارجية</v>
+        <v>مؤشّر المخاطر</v>
       </c>
       <c r="C226" t="str">
-        <v>Opens the historical imagery archive for a chosen site in a new tab</v>
+        <v>Risk index</v>
       </c>
       <c r="D226" t="str">
         <v/>
@@ -8718,10 +8718,10 @@
         <v>T226</v>
       </c>
       <c r="B227" t="str">
-        <v>اختر موقعاً من القائمة أو ابحث، ثم اضغط لفتح الأرشيف التاريخي لمكانه.</v>
+        <v>امسح الرمز للوصول السريع لصفحة هذا الأصل التراثي، أو شارك الرابط مع الجهات المعنية.</v>
       </c>
       <c r="C227" t="str">
-        <v>Pick a site below, or search, then open its historical archive.</v>
+        <v>Scan to quickly access this heritage asset page, or share the link with relevant authorities.</v>
       </c>
       <c r="D227" t="str">
         <v/>
@@ -8738,10 +8738,10 @@
         <v>T227</v>
       </c>
       <c r="B228" t="str">
-        <v>ابحث باسم الموقع…</v>
+        <v>بطاقة أصل تراثي</v>
       </c>
       <c r="C228" t="str">
-        <v>Search by site name…</v>
+        <v>Heritage Asset Card</v>
       </c>
       <c r="D228" t="str">
         <v/>
@@ -8758,10 +8758,10 @@
         <v>T228</v>
       </c>
       <c r="B229" t="str">
-        <v>الاستعلام المتقدم</v>
+        <v>امسح الرمز للصفحة الكاملة</v>
       </c>
       <c r="C229" t="str">
-        <v>Advanced query builder</v>
+        <v>Scan for full page</v>
       </c>
       <c r="D229" t="str">
         <v/>
@@ -8778,10 +8778,10 @@
         <v>T229</v>
       </c>
       <c r="B230" t="str">
-        <v>اجمع أكثر من شرط في آن واحد لتصفية دقيقة</v>
+        <v>ثابتة</v>
       </c>
       <c r="C230" t="str">
-        <v>Combine multiple conditions for precise filtering</v>
+        <v>fixed</v>
       </c>
       <c r="D230" t="str">
         <v/>
@@ -8798,10 +8798,10 @@
         <v>T230</v>
       </c>
       <c r="B231" t="str">
-        <v>إضافة شرط</v>
+        <v>لا توجد مستندات بعد</v>
       </c>
       <c r="C231" t="str">
-        <v>Add condition</v>
+        <v>No documents yet</v>
       </c>
       <c r="D231" t="str">
         <v/>
@@ -8818,10 +8818,10 @@
         <v>T231</v>
       </c>
       <c r="B232" t="str">
-        <v>تطبيق</v>
+        <v>حذف هذه الصورة؟</v>
       </c>
       <c r="C232" t="str">
-        <v>Apply</v>
+        <v>Delete this photo?</v>
       </c>
       <c r="D232" t="str">
         <v/>
@@ -8838,10 +8838,10 @@
         <v>T232</v>
       </c>
       <c r="B233" t="str">
-        <v>إعادة ضبط</v>
+        <v>حذف هذا المستند؟</v>
       </c>
       <c r="C233" t="str">
-        <v>Reset</v>
+        <v>Delete this document?</v>
       </c>
       <c r="D233" t="str">
         <v/>
@@ -8858,10 +8858,10 @@
         <v>T233</v>
       </c>
       <c r="B234" t="str">
-        <v>نسبة التهدّم %</v>
+        <v>جميع المناطق</v>
       </c>
       <c r="C234" t="str">
-        <v>Decay %</v>
+        <v>All regions</v>
       </c>
       <c r="D234" t="str">
         <v/>
@@ -8878,10 +8878,10 @@
         <v>T234</v>
       </c>
       <c r="B235" t="str">
-        <v>مركز البيانات</v>
+        <v>تقرير الأصول التراثية العمرانية</v>
       </c>
       <c r="C235" t="str">
-        <v>Data Center</v>
+        <v>Urban Heritage Assets Report</v>
       </c>
       <c r="D235" t="str">
         <v/>
@@ -8898,10 +8898,10 @@
         <v>T235</v>
       </c>
       <c r="B236" t="str">
-        <v>لم أجد أي موقع مطابق (${scope}).</v>
+        <v>نطاق التقرير:</v>
       </c>
       <c r="C236" t="str">
-        <v>No sites matched (${scope}).</v>
+        <v>Report scope:</v>
       </c>
       <c r="D236" t="str">
         <v/>
@@ -8910,7 +8910,7 @@
         <v/>
       </c>
       <c r="F236" t="str">
-        <v>ديناميكي — لا تلمس ${...}</v>
+        <v/>
       </c>
     </row>
     <row r="237">
@@ -8918,10 +8918,10 @@
         <v>T236</v>
       </c>
       <c r="B237" t="str">
-        <v>أعلى ${num(top.length)} مواقع خطورة (${scope}) — اضغط أي موقع للانتقال إليه:</v>
+        <v>المناطق</v>
       </c>
       <c r="C237" t="str">
-        <v>Top ${num(top.length)} risky sites (${scope}):</v>
+        <v>Regions</v>
       </c>
       <c r="D237" t="str">
         <v/>
@@ -8930,7 +8930,7 @@
         <v/>
       </c>
       <c r="F237" t="str">
-        <v>ديناميكي — لا تلمس ${...}</v>
+        <v/>
       </c>
     </row>
     <row r="238">
@@ -8938,10 +8938,10 @@
         <v>T237</v>
       </c>
       <c r="B238" t="str">
-        <v>أعلى ${num(Math.min(100,top.length))} موقعاً حسب مؤشّر المخاطر المركّب (تهدّم × أهمية × غياب أعمال)</v>
+        <v>متوسط التهدّم</v>
       </c>
       <c r="C238" t="str">
-        <v>Top ${num(Math.min(100,top.length))} by composite risk</v>
+        <v>Avg deterioration</v>
       </c>
       <c r="D238" t="str">
         <v/>
@@ -8950,7 +8950,7 @@
         <v/>
       </c>
       <c r="F238" t="str">
-        <v>ديناميكي — لا تلمس ${...}</v>
+        <v/>
       </c>
     </row>
     <row r="239">
@@ -8958,10 +8958,10 @@
         <v>T238</v>
       </c>
       <c r="B239" t="str">
-        <v>اعرض المواقع التي يبلغ عمرها كذا سنة فأكثر (${num(withAge)} موقعاً له عمر مسجّل)</v>
+        <v>ملحّة للترميم</v>
       </c>
       <c r="C239" t="str">
-        <v>Show sites at least N years old (${num(withAge)} dated)</v>
+        <v>Urgent restoration</v>
       </c>
       <c r="D239" t="str">
         <v/>
@@ -8970,7 +8970,7 @@
         <v/>
       </c>
       <c r="F239" t="str">
-        <v>ديناميكي — لا تلمس ${...}</v>
+        <v/>
       </c>
     </row>
     <row r="240">
@@ -8978,10 +8978,10 @@
         <v>T239</v>
       </c>
       <c r="B240" t="str">
-        <v>${num(vs.length)} قرية تراثية مكتشفة تلقائياً من أسماء المواقع</v>
+        <v>وثيقة رسمية صادرة عن السجل الوطني للتراث العمراني — هيئة التراث</v>
       </c>
       <c r="C240" t="str">
-        <v>${num(vs.length)} villages auto-detected</v>
+        <v>Official document — National Urban Heritage Register, Heritage Commission</v>
       </c>
       <c r="D240" t="str">
         <v/>
@@ -8990,7 +8990,7 @@
         <v/>
       </c>
       <c r="F240" t="str">
-        <v>ديناميكي — لا تلمس ${...}</v>
+        <v/>
       </c>
     </row>
     <row r="241">
@@ -8998,10 +8998,10 @@
         <v>T240</v>
       </c>
       <c r="B241" t="str">
-        <v>نطاقات حماية ٥٠٠م حول ${num(pts.length)} موقع فئة (أ) — كبّر الخريطة لرؤيتها</v>
+        <v>تقرير منطقة</v>
       </c>
       <c r="C241" t="str">
-        <v>500m buffers on ${num(pts.length)} Class A sites — zoom in</v>
+        <v>Region Profile</v>
       </c>
       <c r="D241" t="str">
         <v/>
@@ -9010,7 +9010,7 @@
         <v/>
       </c>
       <c r="F241" t="str">
-        <v>ديناميكي — لا تلمس ${...}</v>
+        <v/>
       </c>
     </row>
     <row r="242">
@@ -9018,10 +9018,10 @@
         <v>T241</v>
       </c>
       <c r="B242" t="str">
-        <v>مواد "${dvSafe(worst[0])}" تتهدّم أسرع</v>
+        <v>فئات الأهمية</v>
       </c>
       <c r="C242" t="str">
-        <v>"${dvSafe(worst[0])}" material decays faster</v>
+        <v>Significance</v>
       </c>
       <c r="D242" t="str">
         <v/>
@@ -9030,7 +9030,7 @@
         <v/>
       </c>
       <c r="F242" t="str">
-        <v>ديناميكي — لا تلمس ${...}</v>
+        <v/>
       </c>
     </row>
     <row r="243">
@@ -9038,10 +9038,10 @@
         <v>T242</v>
       </c>
       <c r="B243" t="str">
-        <v>${DB.regions[ri]} الأعلى تهدّماً</v>
+        <v>أعلى ١٠ مواقع حسب مؤشّر المخاطر</v>
       </c>
       <c r="C243" t="str">
-        <v>${DB.regions[ri]} has the highest decay</v>
+        <v>Top 10 sites by risk index</v>
       </c>
       <c r="D243" t="str">
         <v/>
@@ -9050,7 +9050,7 @@
         <v/>
       </c>
       <c r="F243" t="str">
-        <v>ديناميكي — لا تلمس ${...}</v>
+        <v/>
       </c>
     </row>
     <row r="244">
@@ -9058,10 +9058,10 @@
         <v>T243</v>
       </c>
       <c r="B244" t="str">
-        <v>متوسط ${Math.round(avg*100)}٪ عبر ${num(n)} موقع موثّق</v>
+        <v>اختر منطقتين على الأقل</v>
       </c>
       <c r="C244" t="str">
-        <v>avg ${Math.round(avg*100)}% across ${num(n)} documented sites</v>
+        <v>Select at least two regions</v>
       </c>
       <c r="D244" t="str">
         <v/>
@@ -9070,7 +9070,7 @@
         <v/>
       </c>
       <c r="F244" t="str">
-        <v>ديناميكي — لا تلمس ${...}</v>
+        <v/>
       </c>
     </row>
     <row r="245">
@@ -9078,10 +9078,10 @@
         <v>T244</v>
       </c>
       <c r="B245" t="str">
-        <v>${pct}٪ من مواقع الفئة (أ) (${num(aTotal)} موقع) بلا أعمال ترميم جارية مسجّلة</v>
+        <v>عدد الأصول</v>
       </c>
       <c r="C245" t="str">
-        <v>${pct}% of Class A sites (${num(aTotal)} total) have no recorded ongoing works</v>
+        <v>Total assets</v>
       </c>
       <c r="D245" t="str">
         <v/>
@@ -9090,7 +9090,7 @@
         <v/>
       </c>
       <c r="F245" t="str">
-        <v>ديناميكي — لا تلمس ${...}</v>
+        <v/>
       </c>
     </row>
     <row r="246">
@@ -9098,10 +9098,10 @@
         <v>T245</v>
       </c>
       <c r="B246" t="str">
-        <v>مجموعات محتملة التكرار (${num(dupSites)} موقع)</v>
+        <v>مبانٍ</v>
       </c>
       <c r="C246" t="str">
-        <v>Likely-duplicate groups (${num(dupSites)} sites)</v>
+        <v>Buildings</v>
       </c>
       <c r="D246" t="str">
         <v/>
@@ -9110,7 +9110,7 @@
         <v/>
       </c>
       <c r="F246" t="str">
-        <v>ديناميكي — لا تلمس ${...}</v>
+        <v/>
       </c>
     </row>
     <row r="247">
@@ -9118,10 +9118,10 @@
         <v>T246</v>
       </c>
       <c r="B247" t="str">
-        <v>+ ${num(dupes.length-20)} مجموعة أخرى — صدّر CSV للقائمة الكاملة</v>
+        <v>مناطق</v>
       </c>
       <c r="C247" t="str">
-        <v>+ ${num(dupes.length-20)} more — export CSV for the full list</v>
+        <v>Zones</v>
       </c>
       <c r="D247" t="str">
         <v/>
@@ -9130,7 +9130,7 @@
         <v/>
       </c>
       <c r="F247" t="str">
-        <v>ديناميكي — لا تلمس ${...}</v>
+        <v/>
       </c>
     </row>
     <row r="248">
@@ -9138,10 +9138,10 @@
         <v>T247</v>
       </c>
       <c r="B248" t="str">
-        <v>صفحة ${num(_sheetPage+1)} من ${num(totalPages)} — ${num(vis.length)} موقع</v>
+        <v>اختر منطقة من الفلاتر أولاً</v>
       </c>
       <c r="C248" t="str">
-        <v>Page ${num(_sheetPage+1)} of ${num(totalPages)} — ${num(vis.length)} sites</v>
+        <v>Select a region from filters first</v>
       </c>
       <c r="D248" t="str">
         <v/>
@@ -9150,7 +9150,7 @@
         <v/>
       </c>
       <c r="F248" t="str">
-        <v>ديناميكي — لا تلمس ${...}</v>
+        <v/>
       </c>
     </row>
     <row r="249">
@@ -9158,10 +9158,10 @@
         <v>T248</v>
       </c>
       <c r="B249" t="str">
-        <v>+ ${num(parsed.length-12)} صف آخر</v>
+        <v>التهدّم %</v>
       </c>
       <c r="C249" t="str">
-        <v>+ ${num(parsed.length-12)} more rows</v>
+        <v>Decay %</v>
       </c>
       <c r="D249" t="str">
         <v/>
@@ -9170,7 +9170,7 @@
         <v/>
       </c>
       <c r="F249" t="str">
-        <v>ديناميكي — لا تلمس ${...}</v>
+        <v/>
       </c>
     </row>
     <row r="250">
@@ -9178,10 +9178,10 @@
         <v>T249</v>
       </c>
       <c r="B250" t="str">
-        <v>استيراد ${num(parsed.length-dupCount)} موقع</v>
+        <v>مؤشّر المخاطر</v>
       </c>
       <c r="C250" t="str">
-        <v>Import ${num(parsed.length-dupCount)} sites</v>
+        <v>Risk</v>
       </c>
       <c r="D250" t="str">
         <v/>
@@ -9190,7 +9190,7 @@
         <v/>
       </c>
       <c r="F250" t="str">
-        <v>ديناميكي — لا تلمس ${...}</v>
+        <v/>
       </c>
     </row>
     <row r="251">
@@ -9198,10 +9198,10 @@
         <v>T250</v>
       </c>
       <c r="B251" t="str">
-        <v>✓ تم استيراد ${num(added)} موقع بنجاح</v>
+        <v>خط العرض</v>
       </c>
       <c r="C251" t="str">
-        <v>✓ Imported ${num(added)} sites successfully</v>
+        <v>Latitude</v>
       </c>
       <c r="D251" t="str">
         <v/>
@@ -9210,7 +9210,7 @@
         <v/>
       </c>
       <c r="F251" t="str">
-        <v>ديناميكي — لا تلمس ${...}</v>
+        <v/>
       </c>
     </row>
     <row r="252">
@@ -9218,10 +9218,10 @@
         <v>T251</v>
       </c>
       <c r="B252" t="str">
-        <v>${num(c)} موقع بطراز "${dvSafe(name)}"</v>
+        <v>خط الطول</v>
       </c>
       <c r="C252" t="str">
-        <v>${num(c)} sites with "${dvSafe(name)}" style</v>
+        <v>Longitude</v>
       </c>
       <c r="D252" t="str">
         <v/>
@@ -9230,7 +9230,7 @@
         <v/>
       </c>
       <c r="F252" t="str">
-        <v>ديناميكي — لا تلمس ${...}</v>
+        <v/>
       </c>
     </row>
     <row r="253">
@@ -9238,10 +9238,10 @@
         <v>T252</v>
       </c>
       <c r="B253" t="str">
-        <v>عرض مواقع ${e.ar} فأكثر</v>
+        <v>المواقع التراثية</v>
       </c>
       <c r="C253" t="str">
-        <v>Showing sites ${e.en}+</v>
+        <v>Heritage Sites</v>
       </c>
       <c r="D253" t="str">
         <v/>
@@ -9250,7 +9250,7 @@
         <v/>
       </c>
       <c r="F253" t="str">
-        <v>ديناميكي — لا تلمس ${...}</v>
+        <v/>
       </c>
     </row>
     <row r="254">
@@ -9258,10 +9258,10 @@
         <v>T253</v>
       </c>
       <c r="B254" t="str">
-        <v>النتيجة: ${n} موقع مطابق ضمن الفلتر الحالي</v>
+        <v>المواقع_التراثية</v>
       </c>
       <c r="C254" t="str">
-        <v>Result: ${n} matching sites within current filters</v>
+        <v>heritage_sites</v>
       </c>
       <c r="D254" t="str">
         <v/>
@@ -9270,7 +9270,7 @@
         <v/>
       </c>
       <c r="F254" t="str">
-        <v>ديناميكي — لا تلمس ${...}</v>
+        <v/>
       </c>
     </row>
     <row r="255">
@@ -9278,10 +9278,10 @@
         <v>T254</v>
       </c>
       <c r="B255" t="str">
-        <v>اضغط للتصفية على هذه المنطقة</v>
+        <v>تم تصدير ملف Excel</v>
       </c>
       <c r="C255" t="str">
-        <v>Click to filter by this region</v>
+        <v>Excel file exported</v>
       </c>
       <c r="D255" t="str">
         <v/>
@@ -9298,10 +9298,10 @@
         <v>T255</v>
       </c>
       <c r="B256" t="str">
-        <v>لوحة التحليلات</v>
+        <v>اضغط نقطة أخرى</v>
       </c>
       <c r="C256" t="str">
-        <v>Analytics Dashboard</v>
+        <v>Click another point</v>
       </c>
       <c r="D256" t="str">
         <v/>
@@ -9318,10 +9318,10 @@
         <v>T256</v>
       </c>
       <c r="B257" t="str">
-        <v>تحليل شامل للأصول التراثية المعروضة حالياً</v>
+        <v>م</v>
       </c>
       <c r="C257" t="str">
-        <v>Comprehensive analysis of currently displayed heritage assets</v>
+        <v>m</v>
       </c>
       <c r="D257" t="str">
         <v/>
@@ -9338,10 +9338,10 @@
         <v>T257</v>
       </c>
       <c r="B258" t="str">
-        <v>متوسط نسبة التهدّم</v>
+        <v>المسافة:</v>
       </c>
       <c r="C258" t="str">
-        <v>Average deterioration</v>
+        <v>Distance:</v>
       </c>
       <c r="D258" t="str">
         <v/>
@@ -9358,10 +9358,10 @@
         <v>T258</v>
       </c>
       <c r="B259" t="str">
-        <v>مواقع ملحّة للترميم</v>
+        <v>تم إظهار المطارات على الخريطة</v>
       </c>
       <c r="C259" t="str">
-        <v>Urgent for restoration</v>
+        <v>Airports shown on map</v>
       </c>
       <c r="D259" t="str">
         <v/>
@@ -9378,10 +9378,10 @@
         <v>T259</v>
       </c>
       <c r="B260" t="str">
-        <v>متوسط العمر (سنة)</v>
+        <v>تم إخفاء المطارات</v>
       </c>
       <c r="C260" t="str">
-        <v>Average age (yrs)</v>
+        <v>Airports hidden</v>
       </c>
       <c r="D260" t="str">
         <v/>
@@ -9398,10 +9398,10 @@
         <v>T260</v>
       </c>
       <c r="B261" t="str">
-        <v>مناطق / محافظات</v>
+        <v>* ${num(missDecay)} موقع ينقصه نسبة التهدّم، ${num(missSurvey)} ينقصه الحصر الميداني</v>
       </c>
       <c r="C261" t="str">
-        <v>Regions / governorates</v>
+        <v>* ${num(missDecay)} missing deterioration, ${num(missSurvey)} missing survey</v>
       </c>
       <c r="D261" t="str">
         <v/>
@@ -9410,7 +9410,7 @@
         <v/>
       </c>
       <c r="F261" t="str">
-        <v/>
+        <v>ديناميكي — لا تلمس ${...}</v>
       </c>
     </row>
     <row r="262">
@@ -9418,10 +9418,10 @@
         <v>T261</v>
       </c>
       <c r="B262" t="str">
-        <v>التوزيع حسب المنطقة</v>
+        <v>${num(vis.length)} أصل تراثي</v>
       </c>
       <c r="C262" t="str">
-        <v>Distribution by region</v>
+        <v>${num(vis.length)} heritage assets</v>
       </c>
       <c r="D262" t="str">
         <v/>
@@ -9430,7 +9430,7 @@
         <v/>
       </c>
       <c r="F262" t="str">
-        <v/>
+        <v>ديناميكي — لا تلمس ${...}</v>
       </c>
     </row>
     <row r="263">
@@ -9438,10 +9438,10 @@
         <v>T262</v>
       </c>
       <c r="B263" t="str">
-        <v>فئة الأهمية</v>
+        <v>* عُرضت أول ${num(cap)} موقع من إجمالي ${num(total)}. للحصول على القائمة الكاملة استخدم تصدير CSV.</v>
       </c>
       <c r="C263" t="str">
-        <v>Significance class</v>
+        <v>* Showing first ${num(cap)} of ${num(total)}. Use CSV export for the full list.</v>
       </c>
       <c r="D263" t="str">
         <v/>
@@ -9450,7 +9450,7 @@
         <v/>
       </c>
       <c r="F263" t="str">
-        <v/>
+        <v>ديناميكي — لا تلمس ${...}</v>
       </c>
     </row>
     <row r="264">
@@ -9458,10 +9458,10 @@
         <v>T263</v>
       </c>
       <c r="B264" t="str">
-        <v>مبنى</v>
+        <v>لا توجد مواقع ضمن ${num(radiusKm)} كم</v>
       </c>
       <c r="C264" t="str">
-        <v>buildings</v>
+        <v>No sites within ${num(radiusKm)} km</v>
       </c>
       <c r="D264" t="str">
         <v/>
@@ -9470,7 +9470,7 @@
         <v/>
       </c>
       <c r="F264" t="str">
-        <v/>
+        <v>ديناميكي — لا تلمس ${...}</v>
       </c>
     </row>
     <row r="265">
@@ -9478,10 +9478,10 @@
         <v>T264</v>
       </c>
       <c r="B265" t="str">
-        <v>منطقة</v>
+        <v>${num(near.length)} موقع ضمن ${num(radiusKm)} كم</v>
       </c>
       <c r="C265" t="str">
-        <v>zones</v>
+        <v>${num(near.length)} sites within ${num(radiusKm)} km</v>
       </c>
       <c r="D265" t="str">
         <v/>
@@ -9490,7 +9490,7 @@
         <v/>
       </c>
       <c r="F265" t="str">
-        <v/>
+        <v>ديناميكي — لا تلمس ${...}</v>
       </c>
     </row>
     <row r="266">
@@ -9498,10 +9498,10 @@
         <v>T265</v>
       </c>
       <c r="B266" t="str">
-        <v>أعلى ١٠ محافظات</v>
+        <v>مساجد</v>
       </c>
       <c r="C266" t="str">
-        <v>Top 10 governorates</v>
+        <v>Mosques</v>
       </c>
       <c r="D266" t="str">
         <v/>
@@ -9518,10 +9518,10 @@
         <v>T266</v>
       </c>
       <c r="B267" t="str">
-        <v>نوع التراث</v>
+        <v>أبراج</v>
       </c>
       <c r="C267" t="str">
-        <v>Heritage type</v>
+        <v>Towers</v>
       </c>
       <c r="D267" t="str">
         <v/>
@@ -9538,10 +9538,10 @@
         <v>T267</v>
       </c>
       <c r="B268" t="str">
-        <v>مؤشّر اكتمال البيانات</v>
+        <v>حصون وقلاع</v>
       </c>
       <c r="C268" t="str">
-        <v>Data completeness</v>
+        <v>Forts &amp; castles</v>
       </c>
       <c r="D268" t="str">
         <v/>
@@ -9558,10 +9558,10 @@
         <v>T268</v>
       </c>
       <c r="B269" t="str">
-        <v>نسبة التهدّم</v>
+        <v>قصور</v>
       </c>
       <c r="C269" t="str">
-        <v>Deterioration %</v>
+        <v>Palaces</v>
       </c>
       <c r="D269" t="str">
         <v/>
@@ -9578,10 +9578,10 @@
         <v>T269</v>
       </c>
       <c r="B270" t="str">
-        <v>العمر التقريبي</v>
+        <v>آبار وبرك</v>
       </c>
       <c r="C270" t="str">
-        <v>Approx. age</v>
+        <v>Wells</v>
       </c>
       <c r="D270" t="str">
         <v/>
@@ -9598,10 +9598,10 @@
         <v>T270</v>
       </c>
       <c r="B271" t="str">
-        <v>رقم القرار</v>
+        <v>مبانٍ سكنية</v>
       </c>
       <c r="C271" t="str">
-        <v>Decision no.</v>
+        <v>Residential</v>
       </c>
       <c r="D271" t="str">
         <v/>
@@ -9618,10 +9618,10 @@
         <v>T271</v>
       </c>
       <c r="B272" t="str">
-        <v>بيانات الحصر الميداني</v>
+        <v>قرى وبلدات</v>
       </c>
       <c r="C272" t="str">
-        <v>Field survey data</v>
+        <v>Villages</v>
       </c>
       <c r="D272" t="str">
         <v/>
@@ -9638,10 +9638,10 @@
         <v>T272</v>
       </c>
       <c r="B273" t="str">
-        <v>لا توجد نتائج</v>
+        <v>أحياء ومراكز</v>
       </c>
       <c r="C273" t="str">
-        <v>No results</v>
+        <v>Districts</v>
       </c>
       <c r="D273" t="str">
         <v/>
@@ -9658,10 +9658,10 @@
         <v>T273</v>
       </c>
       <c r="B274" t="str">
-        <v>عرض المزيد</v>
+        <v>مدارس</v>
       </c>
       <c r="C274" t="str">
-        <v>Show more</v>
+        <v>Schools</v>
       </c>
       <c r="D274" t="str">
         <v/>
@@ -9678,10 +9678,10 @@
         <v>T274</v>
       </c>
       <c r="B275" t="str">
-        <v>نهاية القائمة</v>
+        <v>أسواق ومتاجر</v>
       </c>
       <c r="C275" t="str">
-        <v>End of list</v>
+        <v>Markets</v>
       </c>
       <c r="D275" t="str">
         <v/>
@@ -9698,10 +9698,10 @@
         <v>T275</v>
       </c>
       <c r="B276" t="str">
-        <v>أصل</v>
+        <v>أخرى</v>
       </c>
       <c r="C276" t="str">
-        <v>assets</v>
+        <v>Other</v>
       </c>
       <c r="D276" t="str">
         <v/>
@@ -9718,10 +9718,10 @@
         <v>T276</v>
       </c>
       <c r="B277" t="str">
-        <v>لا توجد نتائج مطابقة</v>
+        <v>أقل من ٢٠٪</v>
       </c>
       <c r="C277" t="str">
-        <v>No matching results</v>
+        <v>&lt; 20%</v>
       </c>
       <c r="D277" t="str">
         <v/>
@@ -9738,10 +9738,10 @@
         <v>T277</v>
       </c>
       <c r="B278" t="str">
-        <v>امسح الرمز للوصول السريع لصفحة هذا الأصل التراثي، أو شارك الرابط مع الجهات المعنية.</v>
+        <v>٢٠٪ – ٣٤٪</v>
       </c>
       <c r="C278" t="str">
-        <v>Scan to quickly access this heritage asset page, or share the link with relevant authorities.</v>
+        <v>20–34%</v>
       </c>
       <c r="D278" t="str">
         <v/>
@@ -9758,10 +9758,10 @@
         <v>T278</v>
       </c>
       <c r="B279" t="str">
-        <v>بطاقة أصل تراثي</v>
+        <v>٣٥٪ – ٤٩٪</v>
       </c>
       <c r="C279" t="str">
-        <v>Heritage Asset Card</v>
+        <v>35–49%</v>
       </c>
       <c r="D279" t="str">
         <v/>
@@ -9778,10 +9778,10 @@
         <v>T279</v>
       </c>
       <c r="B280" t="str">
-        <v>امسح الرمز للصفحة الكاملة</v>
+        <v>٥٠٪ فأكثر</v>
       </c>
       <c r="C280" t="str">
-        <v>Scan for full page</v>
+        <v>≥ 50%</v>
       </c>
       <c r="D280" t="str">
         <v/>
@@ -9798,10 +9798,10 @@
         <v>T280</v>
       </c>
       <c r="B281" t="str">
-        <v>ثابتة</v>
+        <v>المساعد الذكي</v>
       </c>
       <c r="C281" t="str">
-        <v>fixed</v>
+        <v>Smart assistant</v>
       </c>
       <c r="D281" t="str">
         <v/>
@@ -9818,10 +9818,10 @@
         <v>T281</v>
       </c>
       <c r="B282" t="str">
-        <v>لا توجد مستندات بعد</v>
+        <v>النمذجة المستقبلية</v>
       </c>
       <c r="C282" t="str">
-        <v>No documents yet</v>
+        <v>Decay projection</v>
       </c>
       <c r="D282" t="str">
         <v/>
@@ -9838,10 +9838,10 @@
         <v>T282</v>
       </c>
       <c r="B283" t="str">
-        <v>حذف هذه الصورة؟</v>
+        <v>مؤشّر صحة التراث</v>
       </c>
       <c r="C283" t="str">
-        <v>Delete this photo?</v>
+        <v>Heritage health index</v>
       </c>
       <c r="D283" t="str">
         <v/>
@@ -9858,10 +9858,10 @@
         <v>T283</v>
       </c>
       <c r="B284" t="str">
-        <v>حذف هذا المستند؟</v>
+        <v>الأولويات الوطنية</v>
       </c>
       <c r="C284" t="str">
-        <v>Delete this document?</v>
+        <v>National priorities</v>
       </c>
       <c r="D284" t="str">
         <v/>
@@ -9878,10 +9878,10 @@
         <v>T284</v>
       </c>
       <c r="B285" t="str">
-        <v>جميع المناطق</v>
+        <v>الخط الزمني</v>
       </c>
       <c r="C285" t="str">
-        <v>All regions</v>
+        <v>Timeline</v>
       </c>
       <c r="D285" t="str">
         <v/>
@@ -9898,10 +9898,10 @@
         <v>T285</v>
       </c>
       <c r="B286" t="str">
-        <v>تقرير الأصول التراثية العمرانية</v>
+        <v>مستكشف القرى</v>
       </c>
       <c r="C286" t="str">
-        <v>Urban Heritage Assets Report</v>
+        <v>Village explorer</v>
       </c>
       <c r="D286" t="str">
         <v/>
@@ -9918,10 +9918,10 @@
         <v>T286</v>
       </c>
       <c r="B287" t="str">
-        <v>نطاق التقرير:</v>
+        <v>المسارات السياحية</v>
       </c>
       <c r="C287" t="str">
-        <v>Report scope:</v>
+        <v>Tourist routes</v>
       </c>
       <c r="D287" t="str">
         <v/>
@@ -9938,10 +9938,10 @@
         <v>T287</v>
       </c>
       <c r="B288" t="str">
-        <v>المناطق</v>
+        <v>جولة سينمائية</v>
       </c>
       <c r="C288" t="str">
-        <v>Regions</v>
+        <v>Cinematic tour</v>
       </c>
       <c r="D288" t="str">
         <v/>
@@ -9958,10 +9958,10 @@
         <v>T288</v>
       </c>
       <c r="B289" t="str">
-        <v>وثيقة رسمية صادرة عن السجل الوطني للتراث العمراني — هيئة التراث</v>
+        <v>نطاقات الحماية</v>
       </c>
       <c r="C289" t="str">
-        <v>Official document — National Urban Heritage Register, Heritage Commission</v>
+        <v>Protection buffers</v>
       </c>
       <c r="D289" t="str">
         <v/>
@@ -9978,10 +9978,10 @@
         <v>T289</v>
       </c>
       <c r="B290" t="str">
-        <v>تقرير منطقة</v>
+        <v>مقارنة رادار</v>
       </c>
       <c r="C290" t="str">
-        <v>Region Profile</v>
+        <v>Radar compare</v>
       </c>
       <c r="D290" t="str">
         <v/>
@@ -9998,10 +9998,10 @@
         <v>T290</v>
       </c>
       <c r="B291" t="str">
-        <v>فئات الأهمية</v>
+        <v>اكتمال الحصر</v>
       </c>
       <c r="C291" t="str">
-        <v>Significance</v>
+        <v>Survey progress</v>
       </c>
       <c r="D291" t="str">
         <v/>
@@ -10018,10 +10018,10 @@
         <v>T291</v>
       </c>
       <c r="B292" t="str">
-        <v>أعلى ١٠ مواقع حسب مؤشّر المخاطر</v>
+        <v>الأطلس الوطني</v>
       </c>
       <c r="C292" t="str">
-        <v>Top 10 sites by risk index</v>
+        <v>National atlas</v>
       </c>
       <c r="D292" t="str">
         <v/>
@@ -10038,10 +10038,10 @@
         <v>T292</v>
       </c>
       <c r="B293" t="str">
-        <v>اختر منطقتين على الأقل</v>
+        <v>تصدير GeoJSON / KML</v>
       </c>
       <c r="C293" t="str">
-        <v>Select at least two regions</v>
+        <v>GeoJSON / KML export</v>
       </c>
       <c r="D293" t="str">
         <v/>
@@ -10058,10 +10058,10 @@
         <v>T293</v>
       </c>
       <c r="B294" t="str">
-        <v>عدد الأصول</v>
+        <v>تسجيل الجولة كفيديو</v>
       </c>
       <c r="C294" t="str">
-        <v>Total assets</v>
+        <v>Record tour as video</v>
       </c>
       <c r="D294" t="str">
         <v/>
@@ -10078,10 +10078,10 @@
         <v>T294</v>
       </c>
       <c r="B295" t="str">
-        <v>مبانٍ</v>
+        <v>عدسة الزمن</v>
       </c>
       <c r="C295" t="str">
-        <v>Buildings</v>
+        <v>Time lens</v>
       </c>
       <c r="D295" t="str">
         <v/>
@@ -10098,10 +10098,10 @@
         <v>T295</v>
       </c>
       <c r="B296" t="str">
-        <v>مناطق</v>
+        <v>إعادة تشغيل النمو</v>
       </c>
       <c r="C296" t="str">
-        <v>Zones</v>
+        <v>Growth replay</v>
       </c>
       <c r="D296" t="str">
         <v/>
@@ -10118,10 +10118,10 @@
         <v>T296</v>
       </c>
       <c r="B297" t="str">
-        <v>اختر منطقة من الفلاتر أولاً</v>
+        <v>محاكي «ماذا لو رمّمنا؟»</v>
       </c>
       <c r="C297" t="str">
-        <v>Select a region from filters first</v>
+        <v>Restoration what-if</v>
       </c>
       <c r="D297" t="str">
         <v/>
@@ -10138,10 +10138,10 @@
         <v>T297</v>
       </c>
       <c r="B298" t="str">
-        <v>مؤشّر المخاطر</v>
+        <v>قصص القرى التفاعلية</v>
       </c>
       <c r="C298" t="str">
-        <v>Risk</v>
+        <v>Village stories</v>
       </c>
       <c r="D298" t="str">
         <v/>
@@ -10158,10 +10158,10 @@
         <v>T298</v>
       </c>
       <c r="B299" t="str">
-        <v>خط العرض</v>
+        <v>الخريطة العتيقة</v>
       </c>
       <c r="C299" t="str">
-        <v>Latitude</v>
+        <v>Vintage map</v>
       </c>
       <c r="D299" t="str">
         <v/>
@@ -10178,10 +10178,10 @@
         <v>T299</v>
       </c>
       <c r="B300" t="str">
-        <v>خط الطول</v>
+        <v>اللوحات التعريفية</v>
       </c>
       <c r="C300" t="str">
-        <v>Longitude</v>
+        <v>Field plaques</v>
       </c>
       <c r="D300" t="str">
         <v/>
@@ -10198,10 +10198,10 @@
         <v>T300</v>
       </c>
       <c r="B301" t="str">
-        <v>المواقع التراثية</v>
+        <v>الحرارة عبر الزمن</v>
       </c>
       <c r="C301" t="str">
-        <v>Heritage Sites</v>
+        <v>Temporal heat map</v>
       </c>
       <c r="D301" t="str">
         <v/>
@@ -10218,10 +10218,10 @@
         <v>T301</v>
       </c>
       <c r="B302" t="str">
-        <v>المواقع_التراثية</v>
+        <v>خريطتان متزامنتان</v>
       </c>
       <c r="C302" t="str">
-        <v>heritage_sites</v>
+        <v>Dual synced maps</v>
       </c>
       <c r="D302" t="str">
         <v/>
@@ -10238,10 +10238,10 @@
         <v>T302</v>
       </c>
       <c r="B303" t="str">
-        <v>تم تصدير ملف Excel</v>
+        <v>اسأل عن البيانات بالعربي</v>
       </c>
       <c r="C303" t="str">
-        <v>Excel file exported</v>
+        <v>Ask the data in plain language</v>
       </c>
       <c r="D303" t="str">
         <v/>
@@ -10258,10 +10258,10 @@
         <v>T303</v>
       </c>
       <c r="B304" t="str">
-        <v>اضغط نقطة أخرى</v>
+        <v>كيف تبدو الخريطة بعد ٢٠ سنة؟</v>
       </c>
       <c r="C304" t="str">
-        <v>Click another point</v>
+        <v>How will the map look in 20 years?</v>
       </c>
       <c r="D304" t="str">
         <v/>
@@ -10278,10 +10278,10 @@
         <v>T304</v>
       </c>
       <c r="B305" t="str">
-        <v>م</v>
+        <v>رقم وطني واحد لحالة التراث</v>
       </c>
       <c r="C305" t="str">
-        <v>m</v>
+        <v>One national score</v>
       </c>
       <c r="D305" t="str">
         <v/>
@@ -10298,10 +10298,10 @@
         <v>T305</v>
       </c>
       <c r="B306" t="str">
-        <v>المسافة:</v>
+        <v>أعلى ١٠٠ موقع استحقاقاً للترميم</v>
       </c>
       <c r="C306" t="str">
-        <v>Distance:</v>
+        <v>Top 100 sites for restoration</v>
       </c>
       <c r="D306" t="str">
         <v/>
@@ -10318,10 +10318,10 @@
         <v>T306</v>
       </c>
       <c r="B307" t="str">
-        <v>تم إظهار المطارات على الخريطة</v>
+        <v>تصفية وعرض المواقع حسب العمر</v>
       </c>
       <c r="C307" t="str">
-        <v>Airports shown on map</v>
+        <v>Filter sites by age</v>
       </c>
       <c r="D307" t="str">
         <v/>
@@ -10338,10 +10338,10 @@
         <v>T307</v>
       </c>
       <c r="B308" t="str">
-        <v>تم إخفاء المطارات</v>
+        <v>ملفات تعريفية للقرى التراثية</v>
       </c>
       <c r="C308" t="str">
-        <v>Airports hidden</v>
+        <v>Heritage village profiles</v>
       </c>
       <c r="D308" t="str">
         <v/>
@@ -10358,10 +10358,10 @@
         <v>T308</v>
       </c>
       <c r="B309" t="str">
-        <v>* ${num(missDecay)} موقع ينقصه نسبة التهدّم، ${num(missSurvey)} ينقصه الحصر الميداني</v>
+        <v>خطّط رحلة بين المواقع القريبة</v>
       </c>
       <c r="C309" t="str">
-        <v>* ${num(missDecay)} missing deterioration, ${num(missSurvey)} missing survey</v>
+        <v>Plan a heritage trip</v>
       </c>
       <c r="D309" t="str">
         <v/>
@@ -10370,7 +10370,7 @@
         <v/>
       </c>
       <c r="F309" t="str">
-        <v>ديناميكي — لا تلمس ${...}</v>
+        <v/>
       </c>
     </row>
     <row r="310">
@@ -10378,10 +10378,10 @@
         <v>T309</v>
       </c>
       <c r="B310" t="str">
-        <v>${num(vis.length)} أصل تراثي</v>
+        <v>طيران تلقائي بين أجمل القرى</v>
       </c>
       <c r="C310" t="str">
-        <v>${num(vis.length)} heritage assets</v>
+        <v>Auto-fly between top villages</v>
       </c>
       <c r="D310" t="str">
         <v/>
@@ -10390,7 +10390,7 @@
         <v/>
       </c>
       <c r="F310" t="str">
-        <v>ديناميكي — لا تلمس ${...}</v>
+        <v/>
       </c>
     </row>
     <row r="311">
@@ -10398,10 +10398,10 @@
         <v>T310</v>
       </c>
       <c r="B311" t="str">
-        <v>* عُرضت أول ${num(cap)} موقع من إجمالي ${num(total)}. للحصول على القائمة الكاملة استخدم تصدير CSV.</v>
+        <v>دوائر ٥٠٠م حول مواقع الفئة (أ)</v>
       </c>
       <c r="C311" t="str">
-        <v>* Showing first ${num(cap)} of ${num(total)}. Use CSV export for the full list.</v>
+        <v>500m buffers around Class A</v>
       </c>
       <c r="D311" t="str">
         <v/>
@@ -10410,7 +10410,7 @@
         <v/>
       </c>
       <c r="F311" t="str">
-        <v>ديناميكي — لا تلمس ${...}</v>
+        <v/>
       </c>
     </row>
     <row r="312">
@@ -10418,10 +10418,10 @@
         <v>T311</v>
       </c>
       <c r="B312" t="str">
-        <v>لا توجد مواقع ضمن ${num(radiusKm)} كم</v>
+        <v>مقارنة المناطق على ٦ محاور</v>
       </c>
       <c r="C312" t="str">
-        <v>No sites within ${num(radiusKm)} km</v>
+        <v>Compare regions on 6 axes</v>
       </c>
       <c r="D312" t="str">
         <v/>
@@ -10430,7 +10430,7 @@
         <v/>
       </c>
       <c r="F312" t="str">
-        <v>ديناميكي — لا تلمس ${...}</v>
+        <v/>
       </c>
     </row>
     <row r="313">
@@ -10438,10 +10438,10 @@
         <v>T312</v>
       </c>
       <c r="B313" t="str">
-        <v>${num(near.length)} موقع ضمن ${num(radiusKm)} كم</v>
+        <v>نسبة اكتمال البيانات لكل منطقة</v>
       </c>
       <c r="C313" t="str">
-        <v>${num(near.length)} sites within ${num(radiusKm)} km</v>
+        <v>Data completeness per region</v>
       </c>
       <c r="D313" t="str">
         <v/>
@@ -10450,7 +10450,7 @@
         <v/>
       </c>
       <c r="F313" t="str">
-        <v>ديناميكي — لا تلمس ${...}</v>
+        <v/>
       </c>
     </row>
     <row r="314">
@@ -10458,10 +10458,10 @@
         <v>T313</v>
       </c>
       <c r="B314" t="str">
-        <v>مساجد</v>
+        <v>تقرير شامل لكل المناطق (طباعة)</v>
       </c>
       <c r="C314" t="str">
-        <v>Mosques</v>
+        <v>Print-ready all-regions report</v>
       </c>
       <c r="D314" t="str">
         <v/>
@@ -10478,10 +10478,10 @@
         <v>T314</v>
       </c>
       <c r="B315" t="str">
-        <v>أبراج</v>
+        <v>افتح بياناتك في Google Earth و QGIS</v>
       </c>
       <c r="C315" t="str">
-        <v>Towers</v>
+        <v>Open your data in GIS tools</v>
       </c>
       <c r="D315" t="str">
         <v/>
@@ -10498,10 +10498,10 @@
         <v>T315</v>
       </c>
       <c r="B316" t="str">
-        <v>حصون وقلاع</v>
+        <v>توثيق كل إضافة وتعديل</v>
       </c>
       <c r="C316" t="str">
-        <v>Forts &amp; castles</v>
+        <v>Every change, documented</v>
       </c>
       <c r="D316" t="str">
         <v/>
@@ -10518,10 +10518,10 @@
         <v>T316</v>
       </c>
       <c r="B317" t="str">
-        <v>قصور</v>
+        <v>فيديو WebM حقيقي للطيران بين القرى</v>
       </c>
       <c r="C317" t="str">
-        <v>Palaces</v>
+        <v>A real downloadable flyover video</v>
       </c>
       <c r="D317" t="str">
         <v/>
@@ -10538,10 +10538,10 @@
         <v>T317</v>
       </c>
       <c r="B318" t="str">
-        <v>آبار وبرك</v>
+        <v>داخل العدسة ٢٠٤٦ وخارجها اليوم</v>
       </c>
       <c r="C318" t="str">
-        <v>Wells</v>
+        <v>Inside: 2046 · outside: today</v>
       </c>
       <c r="D318" t="str">
         <v/>
@@ -10558,10 +10558,10 @@
         <v>T318</v>
       </c>
       <c r="B319" t="str">
-        <v>مبانٍ سكنية</v>
+        <v>شاهد السجل يمتلئ من صفر إلى ٢٠,٨٠٠</v>
       </c>
       <c r="C319" t="str">
-        <v>Residential</v>
+        <v>Watch the register fill 0 → 20,800</v>
       </c>
       <c r="D319" t="str">
         <v/>
@@ -10578,10 +10578,10 @@
         <v>T319</v>
       </c>
       <c r="B320" t="str">
-        <v>قرى وبلدات</v>
+        <v>كم يقفز المؤشر الوطني لو رمّمنا؟</v>
       </c>
       <c r="C320" t="str">
-        <v>Villages</v>
+        <v>How much does the index jump?</v>
       </c>
       <c r="D320" t="str">
         <v/>
@@ -10598,10 +10598,10 @@
         <v>T320</v>
       </c>
       <c r="B321" t="str">
-        <v>أحياء ومراكز</v>
+        <v>رحلة سردية فصولها مبانٍ حقيقية</v>
       </c>
       <c r="C321" t="str">
-        <v>Districts</v>
+        <v>A scrollytelling journey per village</v>
       </c>
       <c r="D321" t="str">
         <v/>
@@ -10618,10 +10618,10 @@
         <v>T321</v>
       </c>
       <c r="B322" t="str">
-        <v>مدارس</v>
+        <v>طراز مخطوطة قديمة بضغطة زر</v>
       </c>
       <c r="C322" t="str">
-        <v>Schools</v>
+        <v>Old-manuscript map skin</v>
       </c>
       <c r="D322" t="str">
         <v/>
@@ -10638,10 +10638,10 @@
         <v>T322</v>
       </c>
       <c r="B323" t="str">
-        <v>أسواق ومتاجر</v>
+        <v>لوحات وملصقات QR جاهزة للطباعة</v>
       </c>
       <c r="C323" t="str">
-        <v>Markets</v>
+        <v>Print-ready QR plaques &amp; labels</v>
       </c>
       <c r="D323" t="str">
         <v/>
@@ -10658,10 +10658,10 @@
         <v>T323</v>
       </c>
       <c r="B324" t="str">
-        <v>أخرى</v>
+        <v>كثافة المواقع تتشكل حسب العمر</v>
       </c>
       <c r="C324" t="str">
-        <v>Other</v>
+        <v>Density blooming through the ages</v>
       </c>
       <c r="D324" t="str">
         <v/>
@@ -10678,10 +10678,10 @@
         <v>T324</v>
       </c>
       <c r="B325" t="str">
-        <v>أقل من ٢٠٪</v>
+        <v>قارن منطقتين جنباً إلى جنب</v>
       </c>
       <c r="C325" t="str">
-        <v>&lt; 20%</v>
+        <v>Compare two regions side-by-side</v>
       </c>
       <c r="D325" t="str">
         <v/>
@@ -10698,10 +10698,10 @@
         <v>T325</v>
       </c>
       <c r="B326" t="str">
-        <v>٢٠٪ – ٣٤٪</v>
+        <v>استورد مواقع من CSV بضغطة واحدة</v>
       </c>
       <c r="C326" t="str">
-        <v>20–34%</v>
+        <v>Import sites from CSV in one click</v>
       </c>
       <c r="D326" t="str">
         <v/>
@@ -10718,10 +10718,10 @@
         <v>T326</v>
       </c>
       <c r="B327" t="str">
-        <v>٣٥٪ – ٤٩٪</v>
+        <v>لقطات مؤشرات وتغيّر عبر الزمن</v>
       </c>
       <c r="C327" t="str">
-        <v>35–49%</v>
+        <v>Stat snapshots over time</v>
       </c>
       <c r="D327" t="str">
         <v/>
@@ -10738,10 +10738,10 @@
         <v>T327</v>
       </c>
       <c r="B328" t="str">
-        <v>٥٠٪ فأكثر</v>
+        <v>الفئة (أ) — أهمية عالية</v>
       </c>
       <c r="C328" t="str">
-        <v>≥ 50%</v>
+        <v>Class A — High value</v>
       </c>
       <c r="D328" t="str">
         <v/>
@@ -10758,10 +10758,10 @@
         <v>T328</v>
       </c>
       <c r="B329" t="str">
-        <v>المساعد الذكي</v>
+        <v>الفئة (ب) — أهمية متوسطة</v>
       </c>
       <c r="C329" t="str">
-        <v>Smart assistant</v>
+        <v>Class B — Medium value</v>
       </c>
       <c r="D329" t="str">
         <v/>
@@ -10778,10 +10778,10 @@
         <v>T329</v>
       </c>
       <c r="B330" t="str">
-        <v>النمذجة المستقبلية</v>
+        <v>الفئة (ج) — أهمية قليلة</v>
       </c>
       <c r="C330" t="str">
-        <v>Decay projection</v>
+        <v>Class C — Lower value</v>
       </c>
       <c r="D330" t="str">
         <v/>
@@ -10798,10 +10798,10 @@
         <v>T330</v>
       </c>
       <c r="B331" t="str">
-        <v>مؤشّر صحة التراث</v>
+        <v>غير مصنّف</v>
       </c>
       <c r="C331" t="str">
-        <v>Heritage health index</v>
+        <v>Unclassified</v>
       </c>
       <c r="D331" t="str">
         <v/>
@@ -10810,1172 +10810,12 @@
         <v/>
       </c>
       <c r="F331" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="332">
-      <c r="A332" t="str">
-        <v>T331</v>
-      </c>
-      <c r="B332" t="str">
-        <v>الأولويات الوطنية</v>
-      </c>
-      <c r="C332" t="str">
-        <v>National priorities</v>
-      </c>
-      <c r="D332" t="str">
-        <v/>
-      </c>
-      <c r="E332" t="str">
-        <v/>
-      </c>
-      <c r="F332" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="333">
-      <c r="A333" t="str">
-        <v>T332</v>
-      </c>
-      <c r="B333" t="str">
-        <v>الخط الزمني</v>
-      </c>
-      <c r="C333" t="str">
-        <v>Timeline</v>
-      </c>
-      <c r="D333" t="str">
-        <v/>
-      </c>
-      <c r="E333" t="str">
-        <v/>
-      </c>
-      <c r="F333" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="334">
-      <c r="A334" t="str">
-        <v>T333</v>
-      </c>
-      <c r="B334" t="str">
-        <v>مستكشف القرى</v>
-      </c>
-      <c r="C334" t="str">
-        <v>Village explorer</v>
-      </c>
-      <c r="D334" t="str">
-        <v/>
-      </c>
-      <c r="E334" t="str">
-        <v/>
-      </c>
-      <c r="F334" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="335">
-      <c r="A335" t="str">
-        <v>T334</v>
-      </c>
-      <c r="B335" t="str">
-        <v>المسارات السياحية</v>
-      </c>
-      <c r="C335" t="str">
-        <v>Tourist routes</v>
-      </c>
-      <c r="D335" t="str">
-        <v/>
-      </c>
-      <c r="E335" t="str">
-        <v/>
-      </c>
-      <c r="F335" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="336">
-      <c r="A336" t="str">
-        <v>T335</v>
-      </c>
-      <c r="B336" t="str">
-        <v>جولة سينمائية</v>
-      </c>
-      <c r="C336" t="str">
-        <v>Cinematic tour</v>
-      </c>
-      <c r="D336" t="str">
-        <v/>
-      </c>
-      <c r="E336" t="str">
-        <v/>
-      </c>
-      <c r="F336" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="337">
-      <c r="A337" t="str">
-        <v>T336</v>
-      </c>
-      <c r="B337" t="str">
-        <v>نطاقات الحماية</v>
-      </c>
-      <c r="C337" t="str">
-        <v>Protection buffers</v>
-      </c>
-      <c r="D337" t="str">
-        <v/>
-      </c>
-      <c r="E337" t="str">
-        <v/>
-      </c>
-      <c r="F337" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="338">
-      <c r="A338" t="str">
-        <v>T337</v>
-      </c>
-      <c r="B338" t="str">
-        <v>مقارنة رادار</v>
-      </c>
-      <c r="C338" t="str">
-        <v>Radar compare</v>
-      </c>
-      <c r="D338" t="str">
-        <v/>
-      </c>
-      <c r="E338" t="str">
-        <v/>
-      </c>
-      <c r="F338" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="339">
-      <c r="A339" t="str">
-        <v>T338</v>
-      </c>
-      <c r="B339" t="str">
-        <v>اكتمال الحصر</v>
-      </c>
-      <c r="C339" t="str">
-        <v>Survey progress</v>
-      </c>
-      <c r="D339" t="str">
-        <v/>
-      </c>
-      <c r="E339" t="str">
-        <v/>
-      </c>
-      <c r="F339" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="340">
-      <c r="A340" t="str">
-        <v>T339</v>
-      </c>
-      <c r="B340" t="str">
-        <v>الأطلس الوطني</v>
-      </c>
-      <c r="C340" t="str">
-        <v>National atlas</v>
-      </c>
-      <c r="D340" t="str">
-        <v/>
-      </c>
-      <c r="E340" t="str">
-        <v/>
-      </c>
-      <c r="F340" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="341">
-      <c r="A341" t="str">
-        <v>T340</v>
-      </c>
-      <c r="B341" t="str">
-        <v>تصدير GeoJSON / KML</v>
-      </c>
-      <c r="C341" t="str">
-        <v>GeoJSON / KML export</v>
-      </c>
-      <c r="D341" t="str">
-        <v/>
-      </c>
-      <c r="E341" t="str">
-        <v/>
-      </c>
-      <c r="F341" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="342">
-      <c r="A342" t="str">
-        <v>T341</v>
-      </c>
-      <c r="B342" t="str">
-        <v>تقدير تكلفة الترميم</v>
-      </c>
-      <c r="C342" t="str">
-        <v>Restoration cost est.</v>
-      </c>
-      <c r="D342" t="str">
-        <v/>
-      </c>
-      <c r="E342" t="str">
-        <v/>
-      </c>
-      <c r="F342" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="343">
-      <c r="A343" t="str">
-        <v>T342</v>
-      </c>
-      <c r="B343" t="str">
-        <v>المخاطر البيئية</v>
-      </c>
-      <c r="C343" t="str">
-        <v>Environmental risk</v>
-      </c>
-      <c r="D343" t="str">
-        <v/>
-      </c>
-      <c r="E343" t="str">
-        <v/>
-      </c>
-      <c r="F343" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="344">
-      <c r="A344" t="str">
-        <v>T343</v>
-      </c>
-      <c r="B344" t="str">
-        <v>موسوعة الطرز</v>
-      </c>
-      <c r="C344" t="str">
-        <v>Style encyclopedia</v>
-      </c>
-      <c r="D344" t="str">
-        <v/>
-      </c>
-      <c r="E344" t="str">
-        <v/>
-      </c>
-      <c r="F344" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="345">
-      <c r="A345" t="str">
-        <v>T344</v>
-      </c>
-      <c r="B345" t="str">
-        <v>العصور التاريخية</v>
-      </c>
-      <c r="C345" t="str">
-        <v>Historical eras</v>
-      </c>
-      <c r="D345" t="str">
-        <v/>
-      </c>
-      <c r="E345" t="str">
-        <v/>
-      </c>
-      <c r="F345" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="346">
-      <c r="A346" t="str">
-        <v>T345</v>
-      </c>
-      <c r="B346" t="str">
-        <v>لوحة القيادة التنفيذية</v>
-      </c>
-      <c r="C346" t="str">
-        <v>Executive one-pager</v>
-      </c>
-      <c r="D346" t="str">
-        <v/>
-      </c>
-      <c r="E346" t="str">
-        <v/>
-      </c>
-      <c r="F346" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="347">
-      <c r="A347" t="str">
-        <v>T346</v>
-      </c>
-      <c r="B347" t="str">
-        <v>مولّد العرض التقديمي</v>
-      </c>
-      <c r="C347" t="str">
-        <v>Slide-deck generator</v>
-      </c>
-      <c r="D347" t="str">
-        <v/>
-      </c>
-      <c r="E347" t="str">
-        <v/>
-      </c>
-      <c r="F347" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="348">
-      <c r="A348" t="str">
-        <v>T347</v>
-      </c>
-      <c r="B348" t="str">
-        <v>صور تاريخية</v>
-      </c>
-      <c r="C348" t="str">
-        <v>Historical imagery</v>
-      </c>
-      <c r="D348" t="str">
-        <v/>
-      </c>
-      <c r="E348" t="str">
-        <v/>
-      </c>
-      <c r="F348" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="349">
-      <c r="A349" t="str">
-        <v>T348</v>
-      </c>
-      <c r="B349" t="str">
-        <v>الاستعلام المتقدم</v>
-      </c>
-      <c r="C349" t="str">
-        <v>Advanced query</v>
-      </c>
-      <c r="D349" t="str">
-        <v/>
-      </c>
-      <c r="E349" t="str">
-        <v/>
-      </c>
-      <c r="F349" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="350">
-      <c r="A350" t="str">
-        <v>T349</v>
-      </c>
-      <c r="B350" t="str">
-        <v>أكثر من ٢٥٠ سنة</v>
-      </c>
-      <c r="C350" t="str">
-        <v>250+ years</v>
-      </c>
-      <c r="D350" t="str">
-        <v/>
-      </c>
-      <c r="E350" t="str">
-        <v/>
-      </c>
-      <c r="F350" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="351">
-      <c r="A351" t="str">
-        <v>T350</v>
-      </c>
-      <c r="B351" t="str">
-        <v>١٥٠ – ٢٤٩ سنة</v>
-      </c>
-      <c r="C351" t="str">
-        <v>150–249 years</v>
-      </c>
-      <c r="D351" t="str">
-        <v/>
-      </c>
-      <c r="E351" t="str">
-        <v/>
-      </c>
-      <c r="F351" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="352">
-      <c r="A352" t="str">
-        <v>T351</v>
-      </c>
-      <c r="B352" t="str">
-        <v>١٠٠ – ١٤٩ سنة</v>
-      </c>
-      <c r="C352" t="str">
-        <v>100–149 years</v>
-      </c>
-      <c r="D352" t="str">
-        <v/>
-      </c>
-      <c r="E352" t="str">
-        <v/>
-      </c>
-      <c r="F352" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="353">
-      <c r="A353" t="str">
-        <v>T352</v>
-      </c>
-      <c r="B353" t="str">
-        <v>٥٠ – ٩٩ سنة</v>
-      </c>
-      <c r="C353" t="str">
-        <v>50–99 years</v>
-      </c>
-      <c r="D353" t="str">
-        <v/>
-      </c>
-      <c r="E353" t="str">
-        <v/>
-      </c>
-      <c r="F353" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="354">
-      <c r="A354" t="str">
-        <v>T353</v>
-      </c>
-      <c r="B354" t="str">
-        <v>أقل من ٥٠ سنة</v>
-      </c>
-      <c r="C354" t="str">
-        <v>Under 50 years</v>
-      </c>
-      <c r="D354" t="str">
-        <v/>
-      </c>
-      <c r="E354" t="str">
-        <v/>
-      </c>
-      <c r="F354" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="355">
-      <c r="A355" t="str">
-        <v>T354</v>
-      </c>
-      <c r="B355" t="str">
-        <v>اسأل عن البيانات بالعربي</v>
-      </c>
-      <c r="C355" t="str">
-        <v>Ask the data in plain language</v>
-      </c>
-      <c r="D355" t="str">
-        <v/>
-      </c>
-      <c r="E355" t="str">
-        <v/>
-      </c>
-      <c r="F355" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="356">
-      <c r="A356" t="str">
-        <v>T355</v>
-      </c>
-      <c r="B356" t="str">
-        <v>كيف تبدو الخريطة بعد ٢٠ سنة؟</v>
-      </c>
-      <c r="C356" t="str">
-        <v>How will the map look in 20 years?</v>
-      </c>
-      <c r="D356" t="str">
-        <v/>
-      </c>
-      <c r="E356" t="str">
-        <v/>
-      </c>
-      <c r="F356" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="357">
-      <c r="A357" t="str">
-        <v>T356</v>
-      </c>
-      <c r="B357" t="str">
-        <v>رقم وطني واحد لحالة التراث</v>
-      </c>
-      <c r="C357" t="str">
-        <v>One national score</v>
-      </c>
-      <c r="D357" t="str">
-        <v/>
-      </c>
-      <c r="E357" t="str">
-        <v/>
-      </c>
-      <c r="F357" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="358">
-      <c r="A358" t="str">
-        <v>T357</v>
-      </c>
-      <c r="B358" t="str">
-        <v>أعلى ١٠٠ موقع استحقاقاً للترميم</v>
-      </c>
-      <c r="C358" t="str">
-        <v>Top 100 sites for restoration</v>
-      </c>
-      <c r="D358" t="str">
-        <v/>
-      </c>
-      <c r="E358" t="str">
-        <v/>
-      </c>
-      <c r="F358" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="359">
-      <c r="A359" t="str">
-        <v>T358</v>
-      </c>
-      <c r="B359" t="str">
-        <v>تصفية وعرض المواقع حسب العمر</v>
-      </c>
-      <c r="C359" t="str">
-        <v>Filter sites by age</v>
-      </c>
-      <c r="D359" t="str">
-        <v/>
-      </c>
-      <c r="E359" t="str">
-        <v/>
-      </c>
-      <c r="F359" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="360">
-      <c r="A360" t="str">
-        <v>T359</v>
-      </c>
-      <c r="B360" t="str">
-        <v>ملفات تعريفية للقرى التراثية</v>
-      </c>
-      <c r="C360" t="str">
-        <v>Heritage village profiles</v>
-      </c>
-      <c r="D360" t="str">
-        <v/>
-      </c>
-      <c r="E360" t="str">
-        <v/>
-      </c>
-      <c r="F360" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="361">
-      <c r="A361" t="str">
-        <v>T360</v>
-      </c>
-      <c r="B361" t="str">
-        <v>خطّط رحلة بين المواقع القريبة</v>
-      </c>
-      <c r="C361" t="str">
-        <v>Plan a heritage trip</v>
-      </c>
-      <c r="D361" t="str">
-        <v/>
-      </c>
-      <c r="E361" t="str">
-        <v/>
-      </c>
-      <c r="F361" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="362">
-      <c r="A362" t="str">
-        <v>T361</v>
-      </c>
-      <c r="B362" t="str">
-        <v>طيران تلقائي بين أجمل القرى</v>
-      </c>
-      <c r="C362" t="str">
-        <v>Auto-fly between top villages</v>
-      </c>
-      <c r="D362" t="str">
-        <v/>
-      </c>
-      <c r="E362" t="str">
-        <v/>
-      </c>
-      <c r="F362" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="363">
-      <c r="A363" t="str">
-        <v>T362</v>
-      </c>
-      <c r="B363" t="str">
-        <v>دوائر ٥٠٠م حول مواقع الفئة (أ)</v>
-      </c>
-      <c r="C363" t="str">
-        <v>500m buffers around Class A</v>
-      </c>
-      <c r="D363" t="str">
-        <v/>
-      </c>
-      <c r="E363" t="str">
-        <v/>
-      </c>
-      <c r="F363" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="364">
-      <c r="A364" t="str">
-        <v>T363</v>
-      </c>
-      <c r="B364" t="str">
-        <v>مقارنة المناطق على ٦ محاور</v>
-      </c>
-      <c r="C364" t="str">
-        <v>Compare regions on 6 axes</v>
-      </c>
-      <c r="D364" t="str">
-        <v/>
-      </c>
-      <c r="E364" t="str">
-        <v/>
-      </c>
-      <c r="F364" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="365">
-      <c r="A365" t="str">
-        <v>T364</v>
-      </c>
-      <c r="B365" t="str">
-        <v>نسبة اكتمال البيانات لكل منطقة</v>
-      </c>
-      <c r="C365" t="str">
-        <v>Data completeness per region</v>
-      </c>
-      <c r="D365" t="str">
-        <v/>
-      </c>
-      <c r="E365" t="str">
-        <v/>
-      </c>
-      <c r="F365" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="366">
-      <c r="A366" t="str">
-        <v>T365</v>
-      </c>
-      <c r="B366" t="str">
-        <v>تقرير شامل لكل المناطق (طباعة)</v>
-      </c>
-      <c r="C366" t="str">
-        <v>Print-ready all-regions report</v>
-      </c>
-      <c r="D366" t="str">
-        <v/>
-      </c>
-      <c r="E366" t="str">
-        <v/>
-      </c>
-      <c r="F366" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="367">
-      <c r="A367" t="str">
-        <v>T366</v>
-      </c>
-      <c r="B367" t="str">
-        <v>افتح بياناتك في Google Earth و QGIS</v>
-      </c>
-      <c r="C367" t="str">
-        <v>Open your data in GIS tools</v>
-      </c>
-      <c r="D367" t="str">
-        <v/>
-      </c>
-      <c r="E367" t="str">
-        <v/>
-      </c>
-      <c r="F367" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="368">
-      <c r="A368" t="str">
-        <v>T367</v>
-      </c>
-      <c r="B368" t="str">
-        <v>توثيق كل إضافة وتعديل</v>
-      </c>
-      <c r="C368" t="str">
-        <v>Every change, documented</v>
-      </c>
-      <c r="D368" t="str">
-        <v/>
-      </c>
-      <c r="E368" t="str">
-        <v/>
-      </c>
-      <c r="F368" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="369">
-      <c r="A369" t="str">
-        <v>T368</v>
-      </c>
-      <c r="B369" t="str">
-        <v>أنماط مستخرجة آلياً من البيانات</v>
-      </c>
-      <c r="C369" t="str">
-        <v>Patterns mined from the data</v>
-      </c>
-      <c r="D369" t="str">
-        <v/>
-      </c>
-      <c r="E369" t="str">
-        <v/>
-      </c>
-      <c r="F369" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="370">
-      <c r="A370" t="str">
-        <v>T369</v>
-      </c>
-      <c r="B370" t="str">
-        <v>تكرارات وتناقضات وحقول ناقصة</v>
-      </c>
-      <c r="C370" t="str">
-        <v>Duplicates, contradictions, gaps</v>
-      </c>
-      <c r="D370" t="str">
-        <v/>
-      </c>
-      <c r="E370" t="str">
-        <v/>
-      </c>
-      <c r="F370" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="371">
-      <c r="A371" t="str">
-        <v>T370</v>
-      </c>
-      <c r="B371" t="str">
-        <v>تقدير تقريبي لتكلفة الترميم</v>
-      </c>
-      <c r="C371" t="str">
-        <v>Rough budget estimate</v>
-      </c>
-      <c r="D371" t="str">
-        <v/>
-      </c>
-      <c r="E371" t="str">
-        <v/>
-      </c>
-      <c r="F371" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="372">
-      <c r="A372" t="str">
-        <v>T371</v>
-      </c>
-      <c r="B372" t="str">
-        <v>تعديل مباشر داخل جدول تفاعلي</v>
-      </c>
-      <c r="C372" t="str">
-        <v>Inline-editable data grid</v>
-      </c>
-      <c r="D372" t="str">
-        <v/>
-      </c>
-      <c r="E372" t="str">
-        <v/>
-      </c>
-      <c r="F372" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="373">
-      <c r="A373" t="str">
-        <v>T372</v>
-      </c>
-      <c r="B373" t="str">
-        <v>استورد مواقع من CSV بضغطة واحدة</v>
-      </c>
-      <c r="C373" t="str">
-        <v>Import sites from CSV in one click</v>
-      </c>
-      <c r="D373" t="str">
-        <v/>
-      </c>
-      <c r="E373" t="str">
-        <v/>
-      </c>
-      <c r="F373" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="374">
-      <c r="A374" t="str">
-        <v>T373</v>
-      </c>
-      <c r="B374" t="str">
-        <v>لقطات مؤشرات وتغيّر عبر الزمن</v>
-      </c>
-      <c r="C374" t="str">
-        <v>Stat snapshots over time</v>
-      </c>
-      <c r="D374" t="str">
-        <v/>
-      </c>
-      <c r="E374" t="str">
-        <v/>
-      </c>
-      <c r="F374" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="375">
-      <c r="A375" t="str">
-        <v>T374</v>
-      </c>
-      <c r="B375" t="str">
-        <v>قفل محلي بكلمة مرور</v>
-      </c>
-      <c r="C375" t="str">
-        <v>Local passphrase lock</v>
-      </c>
-      <c r="D375" t="str">
-        <v/>
-      </c>
-      <c r="E375" t="str">
-        <v/>
-      </c>
-      <c r="F375" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="376">
-      <c r="A376" t="str">
-        <v>T375</v>
-      </c>
-      <c r="B376" t="str">
-        <v>بيانات جاهزة لأنظمة أخرى</v>
-      </c>
-      <c r="C376" t="str">
-        <v>Data shaped for other systems</v>
-      </c>
-      <c r="D376" t="str">
-        <v/>
-      </c>
-      <c r="E376" t="str">
-        <v/>
-      </c>
-      <c r="F376" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="377">
-      <c r="A377" t="str">
-        <v>T376</v>
-      </c>
-      <c r="B377" t="str">
-        <v>مؤشر تقديري من الارتفاع والموقع</v>
-      </c>
-      <c r="C377" t="str">
-        <v>Estimate from elevation &amp; location</v>
-      </c>
-      <c r="D377" t="str">
-        <v/>
-      </c>
-      <c r="E377" t="str">
-        <v/>
-      </c>
-      <c r="F377" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="378">
-      <c r="A378" t="str">
-        <v>T377</v>
-      </c>
-      <c r="B378" t="str">
-        <v>مرجع الطرز المعمارية في السجل</v>
-      </c>
-      <c r="C378" t="str">
-        <v>Architectural styles reference</v>
-      </c>
-      <c r="D378" t="str">
-        <v/>
-      </c>
-      <c r="E378" t="str">
-        <v/>
-      </c>
-      <c r="F378" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="379">
-      <c r="A379" t="str">
-        <v>T378</v>
-      </c>
-      <c r="B379" t="str">
-        <v>تصفح حسب الحقبة التقديرية</v>
-      </c>
-      <c r="C379" t="str">
-        <v>Browse by approximate era</v>
-      </c>
-      <c r="D379" t="str">
-        <v/>
-      </c>
-      <c r="E379" t="str">
-        <v/>
-      </c>
-      <c r="F379" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="380">
-      <c r="A380" t="str">
-        <v>T379</v>
-      </c>
-      <c r="B380" t="str">
-        <v>شاشة عرض للمسؤولين</v>
-      </c>
-      <c r="C380" t="str">
-        <v>Poster screen for leadership</v>
-      </c>
-      <c r="D380" t="str">
-        <v/>
-      </c>
-      <c r="E380" t="str">
-        <v/>
-      </c>
-      <c r="F380" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="381">
-      <c r="A381" t="str">
-        <v>T380</v>
-      </c>
-      <c r="B381" t="str">
-        <v>شرائح جاهزة من الفلتر الحالي</v>
-      </c>
-      <c r="C381" t="str">
-        <v>Slides built from current filter</v>
-      </c>
-      <c r="D381" t="str">
-        <v/>
-      </c>
-      <c r="E381" t="str">
-        <v/>
-      </c>
-      <c r="F381" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="382">
-      <c r="A382" t="str">
-        <v>T381</v>
-      </c>
-      <c r="B382" t="str">
-        <v>تقرير طباعة لكل محافظة</v>
-      </c>
-      <c r="C382" t="str">
-        <v>Print report per governorate</v>
-      </c>
-      <c r="D382" t="str">
-        <v/>
-      </c>
-      <c r="E382" t="str">
-        <v/>
-      </c>
-      <c r="F382" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="383">
-      <c r="A383" t="str">
-        <v>T382</v>
-      </c>
-      <c r="B383" t="str">
-        <v>الأقل متابعة أو اكتمال بيانات</v>
-      </c>
-      <c r="C383" t="str">
-        <v>Least-tracked / least-complete</v>
-      </c>
-      <c r="D383" t="str">
-        <v/>
-      </c>
-      <c r="E383" t="str">
-        <v/>
-      </c>
-      <c r="F383" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="384">
-      <c r="A384" t="str">
-        <v>T383</v>
-      </c>
-      <c r="B384" t="str">
-        <v>افتح الموقع في أرشيف الأقمار الصناعية</v>
-      </c>
-      <c r="C384" t="str">
-        <v>Open the site in satellite history</v>
-      </c>
-      <c r="D384" t="str">
-        <v/>
-      </c>
-      <c r="E384" t="str">
-        <v/>
-      </c>
-      <c r="F384" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="385">
-      <c r="A385" t="str">
-        <v>T384</v>
-      </c>
-      <c r="B385" t="str">
-        <v>صفّ حسب أكثر من شرط في آن واحد</v>
-      </c>
-      <c r="C385" t="str">
-        <v>Multi-condition filter builder</v>
-      </c>
-      <c r="D385" t="str">
-        <v/>
-      </c>
-      <c r="E385" t="str">
-        <v/>
-      </c>
-      <c r="F385" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="386">
-      <c r="A386" t="str">
-        <v>T385</v>
-      </c>
-      <c r="B386" t="str">
-        <v>الفئة (أ) — أهمية عالية</v>
-      </c>
-      <c r="C386" t="str">
-        <v>Class A — High value</v>
-      </c>
-      <c r="D386" t="str">
-        <v/>
-      </c>
-      <c r="E386" t="str">
-        <v/>
-      </c>
-      <c r="F386" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="387">
-      <c r="A387" t="str">
-        <v>T386</v>
-      </c>
-      <c r="B387" t="str">
-        <v>الفئة (ب) — أهمية متوسطة</v>
-      </c>
-      <c r="C387" t="str">
-        <v>Class B — Medium value</v>
-      </c>
-      <c r="D387" t="str">
-        <v/>
-      </c>
-      <c r="E387" t="str">
-        <v/>
-      </c>
-      <c r="F387" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="388">
-      <c r="A388" t="str">
-        <v>T387</v>
-      </c>
-      <c r="B388" t="str">
-        <v>الفئة (ج) — أهمية قليلة</v>
-      </c>
-      <c r="C388" t="str">
-        <v>Class C — Lower value</v>
-      </c>
-      <c r="D388" t="str">
-        <v/>
-      </c>
-      <c r="E388" t="str">
-        <v/>
-      </c>
-      <c r="F388" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="389">
-      <c r="A389" t="str">
-        <v>T388</v>
-      </c>
-      <c r="B389" t="str">
-        <v>غير مصنّف</v>
-      </c>
-      <c r="C389" t="str">
-        <v>Unclassified</v>
-      </c>
-      <c r="D389" t="str">
-        <v/>
-      </c>
-      <c r="E389" t="str">
-        <v/>
-      </c>
-      <c r="F389" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F389"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F331"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>